<commit_message>
Add verified Ind AS 108 segment tables to Sheet 6 (Phase 2)
Replaced the qualitative segment placeholders with real segment
revenue/results/assets tables extracted from the audited Annual Reports:
- Adani Power: 2 segments (Power Generation; Trading/Investment & other),
  FY20-FY26 series
- Tata Power: 4 segments (Thermal & Hydro, Renewables, T&D, Others),
  FY21-FY26 series, with FY23 restatement and Mundra-shutdown effects noted
- Torrent Power: verified correction - reports NO reportable segments under
  Ind AS 108 (single integrated business; cables immaterial), contrary to
  the earlier 3-segment assumption

Added a segment revenue trend chart and a numbers-based comparative
analysis (Adani dominant in generation; Tata Renewables now its growth
engine; T&D its steadiest earner).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -15,15 +15,16 @@
     <sheet name="4_Acquisitions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="5_Shareholding_Pattern" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="6_Business_Segments" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="7_Group_Structure" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="8_Associates_JVs" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="9_Investments" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="10_Financing_Changes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="11_Returns_Volatility" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Weekly_Price_Data" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="12_Major_Announcements" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="12b_Announcement_Chart_Data" sheetId="16" state="hidden" r:id="rId16"/>
-    <sheet name="13_Sources_and_Gaps" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="6b_Segment_Chart_Data" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet name="7_Group_Structure" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="8_Associates_JVs" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="9_Investments" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="10_Financing_Changes" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="11_Returns_Volatility" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Weekly_Price_Data" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="12_Major_Announcements" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="12b_Announcement_Chart_Data" sheetId="17" state="hidden" r:id="rId17"/>
+    <sheet name="13_Sources_and_Gaps" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -142,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,6 +173,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -732,6 +734,220 @@
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Segment Revenue Trends FY21-FY26 (₹ crore): Tata segments vs Adani Generation</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'6b_Segment_Chart_Data'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$B$2:$B$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'6b_Segment_Chart_Data'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'6b_Segment_Chart_Data'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$D$2:$D$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'6b_Segment_Chart_Data'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'6b_Segment_Chart_Data'!$E$2:$E$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fiscal Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>₹ crore</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="12"/>
   <chart>
     <title>
@@ -834,7 +1050,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -1264,6 +1480,33 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
+      <row>59</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="4680000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
       <row>44</row>
       <rowOff>0</rowOff>
     </from>
@@ -1285,7 +1528,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1811,7 +2054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1823,12 +2066,16 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>8. Associates &amp; Joint Ventures</t>
+          <t>7. Group Structure — Subsidiaries</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr"/>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Key subsidiaries and % holding, with one-line business description.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="5">
@@ -1839,17 +2086,17 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Associate / JV</t>
+          <t>Subsidiary</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Stake</t>
+          <t>% Holding</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Business Description</t>
         </is>
       </c>
     </row>
@@ -1861,17 +2108,17 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Moxie Power Generation Ltd (ex-Coastal Energen, 1,200 MW, Tamil Nadu)</t>
+          <t>Mahan Energen Ltd (MEL)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>49% (JV with Dickey Alternative Investment Trust, 51%)</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Adani does NOT hold majority — classified as JV/associate, not a subsidiary.</t>
+          <t>1,200 MW (2x600) coal thermal plant, MP; ex-Essar Power MP, acquired via CIRP Mar 2022.</t>
         </is>
       </c>
     </row>
@@ -1883,17 +2130,17 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Jaiprakash Power Ventures Ltd (JPVL)</t>
+          <t>Korba Power Ltd (KPL)</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>24% (indirect, via resolution plan)</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Adani Power named 'Implementing Entity'; NCLT-approved ~Mar 2026 (~₹14,535 cr resolution plan).</t>
+          <t>600 MW (2x300) coal thermal plant, Chhattisgarh; ex-Lanco Amarkantak, NCLT-approved Aug 2024.</t>
         </is>
       </c>
     </row>
@@ -1905,105 +2152,501 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Adani Power–Druk Green Power Corp JV (Bhutan)</t>
+          <t>Kutchh Power Generation Ltd (KPGL)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Not disclosed</t>
+          <t>100% (step-down, via APDL)</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>570 MW Wangchhu hydro project (~₹6,000 cr); Shareholders Agreement signed Sep 2025; part of a broader 5,000 MW MoU (May 2025).</t>
+          <t>Held via Adani Power Dahanu Ltd (APDL); generation asset in Gujarat.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Tata Power Delhi Distribution Ltd</t>
+          <t>Adani Power Dahanu Ltd (APDL)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>51% (see Sheet 7 — sometimes classified as JV given 49% Delhi Govt partner)</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Listed here for completeness; treated as subsidiary in Sheet 7 given majority control.</t>
+          <t>Holding vehicle for Dahanu-related generation assets.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Dorjilung Hydro Power Ltd (Bhutan)</t>
+          <t>Adani Atomic Energy Ltd (AAEL)</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Stake not disclosed</t>
+          <t>100% (incorporated Feb 2026)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>1,125 MW hydro project under development.</t>
+          <t>New entry into nuclear power generation, post the SHANTI Act 2025 opening the sector to private players.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>[Other associates/JVs]</t>
+          <t>Progressive-UP Atomic Energy / Coastal-Maha Atomic Energy Ltd (CMAEL)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: Tata Power's full associates/JV list not retrievable via search — pull from Annual Report.</t>
+          <t>100% (step-down, incorporated 2026)</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Further nuclear-energy project SPVs.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
+          <t>Adani Power</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>[6 amalgamated cos: Adani Power Maharashtra, Adani Power Rajasthan, Udupi Power Corp, Raipur Energen, Raigarh Energy Generation, Adani Power (Mundra)]</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>N/A — merged into parent 1-Oct-2021</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Corporate simplification: these erstwhile subsidiaries were amalgamated directly into Adani Power Ltd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>[FULL AOC-1 list]</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>VERIFY: complete statutory subsidiary list with exact % holdings should be pulled from the AOC-1 annexure of the FY23/FY24 Annual Report (BSE corporate filings).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power Renewable Energy Ltd (TPREL)</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>~100% (verify current %)</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Renewable energy arm — utility-scale + rooftop solar and wind generation/EPC; itself has 70 subsidiaries (47 wholly-owned) as of Mar-2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power Solar Systems Ltd (TPSSL)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Verify %</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Solar cell/module manufacturing and EPC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power Delhi Distribution Ltd (Tata Power-DDL)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>51% (JV with Delhi Govt / Delhi Power Co Ltd, 49%)</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Electricity distribution licensee for North Delhi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>TP Northern/Central/Western/Southern Odisha Distribution Ltds (TPNODL/TPCODL/TPWODL/TPSODL)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>51% each</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Four Odisha discoms acquired 2020-21 (PPP with Odisha Govt); serve 12.6mn+ customers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Resurgent Power Ventures Pte Ltd (incl. NRSS XXXVI Transmission Ltd, South East UP Power Transmission Co Ltd)</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Verify %</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Acquisition vehicle for transmission-project SPVs (acquired 2023).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Coastal Gujarat Power Ltd (CGPL) — NOTE</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Merged into parent, 1-Apr-2020</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Owner/operator of Mundra UMPP; NCLT-approved merger means it is NO LONGER a separate subsidiary — Mundra is now a direct Generation-segment asset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>[FULL subsidiary/JV/associate list]</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>VERIFY: Tata Power's 'Subsidiaries, JVs and Associates' annexure (dozens of generation/transmission/renewable SPVs) — pull from the Integrated Annual Report or AOC-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>Torrent Power</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>2 associate companies (per AOC-1 reference)</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Not disclosed</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: names/business of the 2 associate companies not found via search — pull from Annual Report AOC-1.</t>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power Grid Ltd</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>74% (JV; PowerGrid Corp of India holds 26%)</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Interstate power transmission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Pipavav Generation Ltd</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Power generation, Pipavav.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Solargen Ltd</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Solar power generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Jodhpur Wind Farms Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Wind power generation, Rajasthan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Latur Renewable Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Renewable power generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Electricals Pvt Ltd (ex-TCL Cables Pvt Ltd)</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Cables/electricals manufacturing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Dadra &amp; Nagar Haveli and Daman &amp; Diu Power Distribution Corp Ltd</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Power distribution licensee (DNH&amp;DD), acquired 2022.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Nabha Power Ltd</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>100% (acquired Jun 2025)</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>2x700 MW coal-based supercritical thermal plant, Punjab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Visual Percept Solar Projects Pvt Ltd, Surya Vidyut Ltd, Sunshakti Solar Power Projects Pvt Ltd, Torrent Saurya Urja series</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>100% (Torrent Saurya Urja 2 confirmed; others not confirmed %)</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Solar power project SPVs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>[FULL list — ~35 subsidiaries reported]</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>VERIFY: only a partial list could be corroborated; pull the complete AOC-1 statement from torrentpower.com/index.php/site/info/subsidiaries or the Annual Report.</t>
         </is>
       </c>
     </row>
@@ -2022,6 +2665,217 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>8. Associates &amp; Joint Ventures</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr"/>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Associate / JV</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Stake</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Moxie Power Generation Ltd (ex-Coastal Energen, 1,200 MW, Tamil Nadu)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>49% (JV with Dickey Alternative Investment Trust, 51%)</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Adani does NOT hold majority — classified as JV/associate, not a subsidiary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Jaiprakash Power Ventures Ltd (JPVL)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>24% (indirect, via resolution plan)</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power named 'Implementing Entity'; NCLT-approved ~Mar 2026 (~₹14,535 cr resolution plan).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Adani Power–Druk Green Power Corp JV (Bhutan)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>570 MW Wangchhu hydro project (~₹6,000 cr); Shareholders Agreement signed Sep 2025; part of a broader 5,000 MW MoU (May 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power Delhi Distribution Ltd</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>51% (see Sheet 7 — sometimes classified as JV given 49% Delhi Govt partner)</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Listed here for completeness; treated as subsidiary in Sheet 7 given majority control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Dorjilung Hydro Power Ltd (Bhutan)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Stake not disclosed</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>1,125 MW hydro project under development.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Tata Power</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>[Other associates/JVs]</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>VERIFY: Tata Power's full associates/JV list not retrievable via search — pull from Annual Report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Torrent Power</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>2 associate companies (per AOC-1 reference)</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Not disclosed</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>VERIFY: names/business of the 2 associate companies not found via search — pull from Annual Report AOC-1.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2110,7 +2964,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Note: this section requires the 'Investments' note from each company's FY2023 standalone/consolidated Balance Sheet — none of the three companies' figures could be reliably retrieved via web search in this session.</t>
         </is>
@@ -2126,7 +2980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2490,7 +3344,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2524,7 +3378,7 @@
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>HOW TO COMPLETE THIS SHEET</t>
         </is>
@@ -2800,7 +3654,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Key data-quality flag</t>
         </is>
@@ -2848,7 +3702,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3126,7 +3980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3443,7 +4297,7 @@
       <c r="D19" s="11" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Note on this section</t>
         </is>
@@ -3470,7 +4324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3576,7 +4430,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3650,7 +4504,7 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>4. Segment-wise (Ind AS 108) revenue/assets/profit tables, 5-yr, all three companies — pull from the 'Segment Reporting' note in each Annual Report (the PDFs now in the repo contain this — worth a follow-up extraction pass).</t>
+          <t>4. Segment-wise (Ind AS 108) tables — DONE: Sheet 6 now carries verified segment revenue/results/assets for Adani Power (FY20-FY26, 2 segments) and Tata Power (FY21-FY26, 4 segments), plus the verified finding that Torrent Power reports NO segments under Ind AS 108 (single integrated business).</t>
         </is>
       </c>
     </row>
@@ -6488,163 +7342,668 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>6. Reportable Business Segments</t>
+          <t>6. Reportable Business Segments (Ind AS 108) — VERIFIED from Annual Reports</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>As disclosed under Ind AS 108 in each company's Annual Report.</t>
+          <t>₹ crore, consolidated. Extracted directly from the 'Segment Reporting' notes of each company's audited Annual Reports (FY21-FY26 reports uploaded by user).</t>
         </is>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1"/>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr"/>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Reportable segments (per Annual Report)</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Two segments: (1) Power Generation, (2) Trading, Investment &amp; Other activities.</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>~Four segments: (1) Generation, (2) Transmission &amp; Distribution, (3) Renewables, (4) Solar EPC/Manufacturing &amp; Other.</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>Three segments: (1) Generation (gas/coal/renewables), (2) Transmission, (3) Distribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="90" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>ADANI POWER — 2 segments: 'Power Generation &amp; related activities' + 'Trading, Investment &amp; other activities'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>FY20</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>FY21</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>FY22</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Approx. revenue mix (most recent disclosed)</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Power Generation is overwhelmingly dominant; Trading/Other is a small residual. Exact % split not found.</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>T&amp;D ~55% of revenue, Renewables ~25%, remainder Generation + Other/EPC (FY24/25-era mix, qualitative).</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>Distribution is the largest revenue contributor (regulated + volume-driven); Generation dominates capacity but a large share of gas/coal output is sold to the Group's own distribution business.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="90" customHeight="1">
+          <t>Segment Revenue — Power Generation</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>26005.92</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>25870.6</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>27221.78</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>37895.85</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>50014.16</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>56107.06</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>54240.52</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>5-yr segment-wise revenue / assets / profit table</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>NOT FOUND — segment note (Ind AS 108) inside Annual Report notes-to-accounts was inaccessible via search; pull directly from FY19-FY23 Annual Report PDFs.</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>NOT FOUND — same issue; pull the segment-reporting note from each year's Annual Report.</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>NOT FOUND — same issue; only qualitative capacity data (e.g., FY23 distribution electricity purchase +63.2% YoY to 30,037 MU) was found via search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="90" customHeight="1">
+          <t>Segment Revenue — Trading/Investment/Other</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>461.8</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>350.88</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>489.4</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>877.45</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>337.09</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>96.03</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Segment growth vs industry benchmark</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>India's overall power demand grew ~7-8%/yr in recent years (CEA data); Adani Power's generation-segment growth (capacity nearly doubled since FY22 via M&amp;A) has materially outpaced organic sector growth.</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>T&amp;D segment growth benefited from 4 new Odisha discoms (2020-21) — inorganic, faster than organic distribution-sector growth; Renewables segment growing faster than India's ~15-20%/yr renewable capacity addition rate per company commentary.</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Distribution segment volume growth (+63.2% in FY23) was overwhelmingly driven by the DNH&amp;DD acquisition (inorganic), not organic like-for-like growth — strip this out for a fair industry comparison.</t>
-        </is>
+          <t>Segment Results — Power Generation</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>6571.37</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>6957.13</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>20557.22</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>16540.39</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>15757.55</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Segment Results — Trading/Investment/Other</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>717.5700000000001</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>234.29</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>-1.81</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>13.68</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Comparative comment</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="100" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Adani Power is essentially a pure-play generation company (single dominant segment), while Tata Power and Torrent Power are vertically integrated across generation-transmission-distribution, which structurally smooths their earnings (regulated D&amp;T returns cushion merchant-generation volatility) relative to Adani Power's more merchant/PPA-driven, generation-only earnings profile. Among the two integrated peers, Tata Power is furthest along the renewables transition (~25% of revenue mix, explicit 100%-renewable ambition), while Torrent Power remains more gas/coal-weighted in generation with distribution as its largest and most stable segment. A precise, numbers-based segment growth-rate comparison could not be completed — the exact Ind AS 108 segment tables (revenue/assets/profit by segment, 5-yr) need to be manually extracted from each company's Annual Report notes, as this data is not surfaced by web search.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Power Generation</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>74847.53999999999</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>77747</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>81888.09</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>84364.22</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>91378.85000000001</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>111162.48</v>
+      </c>
+      <c r="H11" s="19" t="n">
+        <v>139777.31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Trading/Investment/Other</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>177.46</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>788.47</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>42.02</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1134.26</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>203.86</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>1328.18</v>
+      </c>
+      <c r="H12" s="19" t="n">
+        <v>1354.52</v>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>FY20/21 segment results shown as N/A because the FY21 report used a different basis ('profit before interest…', not comparable); FY22-23 results are as restated in the FY23 report after a CODM methodology change. FY26 Trading revenue was nil; segment results shown are pre-tax basis per each year's note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>TATA POWER — 4 segments: Generation (Thermal &amp; Hydro), Renewables, Transmission &amp; Distribution, Others</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>FY21</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>FY22</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Segment Revenue — Generation/Thermal &amp; Hydro</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>13432.77</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>11211.03</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>18211.35</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>19613.61</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>19739.07</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>11635.93</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Segment Revenue — Renewables</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>5887.65</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>7748.9</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>8196.91</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>10175.29</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>9876.360000000001</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>15027.82</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Segment Revenue — Transmission &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>16829.85</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>27493.17</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>34529.36</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>36205.82</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>39120.52</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>41338.59</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Segment Revenue — Others</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>262.16</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>317.8</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>413.56</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>430.62</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>431.04</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>431.79</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Segment Results — Generation/Thermal &amp; Hydro</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>2709.81</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>2632.75</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>5092.16</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>2569.61</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>2878.91</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>1137.94</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Segment Results — Renewables</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>1494.25</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>1923.57</v>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>1932.01</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>2147.1</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>2880.68</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>4340.93</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Segment Results — Transmission &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>1677.02</v>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>2138.49</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>2197.68</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>2418.22</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>3128.27</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>4307.95</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Segment Results — Others</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>83.16</v>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>-286.03</v>
+      </c>
+      <c r="D24" s="19" t="n">
+        <v>-308.17</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>105.38</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>104.72</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Generation/Thermal &amp; Hydro</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n">
+        <v>37717.32</v>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>38201.93</v>
+      </c>
+      <c r="D25" s="19" t="n">
+        <v>41201.04</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>39315.88</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>39708.11</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>41697.31</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Renewables</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="n">
+        <v>22702.98</v>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>27589.28</v>
+      </c>
+      <c r="D26" s="19" t="n">
+        <v>29744.49</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>40459.25</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>51355.61</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>56921.28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Transmission &amp; Distribution</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="n">
+        <v>25542.61</v>
+      </c>
+      <c r="C27" s="19" t="n">
+        <v>32411.34</v>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>37477.26</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>42059.9</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>45707.75</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>53428.87</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Segment Assets — Others + Unallocable</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>12875.95</v>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>14682.04</v>
+      </c>
+      <c r="D28" s="19" t="n">
+        <v>19926.25</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>17718.46</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>19939.82</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>23124.32</v>
+      </c>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Revenue shown gross (before inter-segment eliminations of ~₹4,000-5,400cr/yr, mostly Generation→T&amp;D coal/power sales). 'Generation' was renamed 'Thermal &amp; Hydro' from the FY25 report. FY23 Generation result of ₹5,092cr was later restated in the FY24 report to ₹1,528cr segment result + ₹3,564cr exceptional; the as-originally-reported figure is shown here. FY26 Thermal &amp; Hydro result derived as total-minus-other-segments (₹9,891.54cr total). FY26 revenue drop in Thermal &amp; Hydro reflects the Mundra shutdown; Renewables surged on new capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>TORRENT POWER — NO reportable segments under Ind AS 108</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="95" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Per Note 53/54 ('Operating Segments') of Torrent Power's FY23 Annual Report (and equivalent notes in other years): "the Group does not have any reportable segment as per Ind AS-108 'Operating Segments'" — the CODM manages Generation, Transmission and Distribution as ONE integrated electricity business, and the cable business is immaterial (below reportable thresholds for revenue, profit and assets). This is an important verified correction: earlier drafts of this sheet assumed 3 reportable segments (Generation/Transmission/Distribution) from the MD&amp;A's business description — the MD&amp;A discusses those businesses operationally, but the statutory segment note reports a single segment. Any segment-level financial comparison for Torrent must therefore rely on MD&amp;A operating metrics (e.g., FY23 distribution electricity purchases +63.2% YoY to 30,037 MU after the DNH&amp;DD takeover), not audited segment P&amp;L data, because none is published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>Comparative analysis — who is doing well in which segment?</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="150" customHeight="1">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>GENERATION is the only segment where all three effectively compete, and the verified numbers show a stark contrast: Adani Power's generation segment grew revenue ~2.1x (₹26,006cr FY20 → ₹54,241cr FY26) with segment results of ₹15,758-20,557cr in FY24-26 — vastly more profitable than Tata Power's generation segment (results of only ₹1,138-2,879cr on ₹11,636-19,739cr revenue in the same years, dragged by the Mundra plant's fuel economics and eventual shutdown). Adani is unambiguously the generation winner. RENEWABLES: only Tata Power reports it separately, and it is now their growth engine — revenue up 2.6x (₹5,888cr FY21 → ₹15,028cr FY26), results up 2.9x (₹1,494cr → ₹4,341cr), and segment assets up 2.5x to ₹56,921cr, overtaking every other Tata segment. Adani Power has no renewables segment (that sits in sister company Adani Green). TRANSMISSION &amp; DISTRIBUTION: Tata Power's largest and steadiest segment — revenue grew ₹16,830cr → ₹41,339cr (FY21→FY26, boosted by the Odisha discoms) with consistently positive, regulated-return results (₹1,677cr → ₹4,308cr). Torrent's distribution business is economically similar (regulated, stable) but not separately reported. INDUSTRY CONTEXT: India's power demand grew ~7-8%/yr (CEA) over this period — Adani's generation growth (~13% CAGR) and Tata's renewables growth (~21% CAGR) both outpaced the sector, largely through acquisitions and capacity build-out respectively, while Tata's generation segment underperformed the sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A12:D18"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="6">
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A39:H47"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A32:H36"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6654,607 +8013,151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>7. Group Structure — Subsidiaries</t>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tata Generation Rev</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Tata Renewables Rev</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Tata T&amp;D Rev</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Adani Generation Rev</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Key subsidiaries and % holding, with one-line business description.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FY21</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>13432.77</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5887.65</v>
+      </c>
+      <c r="D2" t="n">
+        <v>16829.85</v>
+      </c>
+      <c r="E2" t="n">
+        <v>25870.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FY22</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11211.03</v>
+      </c>
+      <c r="C3" t="n">
+        <v>7748.9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>27493.17</v>
+      </c>
+      <c r="E3" t="n">
+        <v>27221.78</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>18211.35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8196.91</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34529.36</v>
+      </c>
+      <c r="E4" t="n">
+        <v>37895.85</v>
+      </c>
+    </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Subsidiary</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>% Holding</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Business Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Mahan Energen Ltd (MEL)</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>1,200 MW (2x600) coal thermal plant, MP; ex-Essar Power MP, acquired via CIRP Mar 2022.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Korba Power Ltd (KPL)</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>600 MW (2x300) coal thermal plant, Chhattisgarh; ex-Lanco Amarkantak, NCLT-approved Aug 2024.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Kutchh Power Generation Ltd (KPGL)</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>100% (step-down, via APDL)</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>Held via Adani Power Dahanu Ltd (APDL); generation asset in Gujarat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power Dahanu Ltd (APDL)</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Holding vehicle for Dahanu-related generation assets.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Adani Atomic Energy Ltd (AAEL)</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>100% (incorporated Feb 2026)</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>New entry into nuclear power generation, post the SHANTI Act 2025 opening the sector to private players.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Progressive-UP Atomic Energy / Coastal-Maha Atomic Energy Ltd (CMAEL)</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>100% (step-down, incorporated 2026)</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>Further nuclear-energy project SPVs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>[6 amalgamated cos: Adani Power Maharashtra, Adani Power Rajasthan, Udupi Power Corp, Raipur Energen, Raigarh Energy Generation, Adani Power (Mundra)]</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>N/A — merged into parent 1-Oct-2021</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>Corporate simplification: these erstwhile subsidiaries were amalgamated directly into Adani Power Ltd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Adani Power</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>[FULL AOC-1 list]</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: complete statutory subsidiary list with exact % holdings should be pulled from the AOC-1 annexure of the FY23/FY24 Annual Report (BSE corporate filings).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power Renewable Energy Ltd (TPREL)</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>~100% (verify current %)</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>Renewable energy arm — utility-scale + rooftop solar and wind generation/EPC; itself has 70 subsidiaries (47 wholly-owned) as of Mar-2024.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power Solar Systems Ltd (TPSSL)</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Verify %</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>Solar cell/module manufacturing and EPC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power Delhi Distribution Ltd (Tata Power-DDL)</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>51% (JV with Delhi Govt / Delhi Power Co Ltd, 49%)</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Electricity distribution licensee for North Delhi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>TP Northern/Central/Western/Southern Odisha Distribution Ltds (TPNODL/TPCODL/TPWODL/TPSODL)</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>51% each</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>Four Odisha discoms acquired 2020-21 (PPP with Odisha Govt); serve 12.6mn+ customers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Resurgent Power Ventures Pte Ltd (incl. NRSS XXXVI Transmission Ltd, South East UP Power Transmission Co Ltd)</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>Verify %</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Acquisition vehicle for transmission-project SPVs (acquired 2023).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Coastal Gujarat Power Ltd (CGPL) — NOTE</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Merged into parent, 1-Apr-2020</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>Owner/operator of Mundra UMPP; NCLT-approved merger means it is NO LONGER a separate subsidiary — Mundra is now a direct Generation-segment asset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Tata Power</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>[FULL subsidiary/JV/associate list]</t>
-        </is>
-      </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: Tata Power's 'Subsidiaries, JVs and Associates' annexure (dozens of generation/transmission/renewable SPVs) — pull from the Integrated Annual Report or AOC-1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power Grid Ltd</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
-        <is>
-          <t>74% (JV; PowerGrid Corp of India holds 26%)</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>Interstate power transmission.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Pipavav Generation Ltd</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>95%</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>Power generation, Pipavav.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Solargen Ltd</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Solar power generation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Jodhpur Wind Farms Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>Wind power generation, Rajasthan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Latur Renewable Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>Renewable power generation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Electricals Pvt Ltd (ex-TCL Cables Pvt Ltd)</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Cables/electricals manufacturing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Dadra &amp; Nagar Haveli and Daman &amp; Diu Power Distribution Corp Ltd</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>51%</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>Power distribution licensee (DNH&amp;DD), acquired 2022.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr">
-        <is>
-          <t>Nabha Power Ltd</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>100% (acquired Jun 2025)</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>2x700 MW coal-based supercritical thermal plant, Punjab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>Visual Percept Solar Projects Pvt Ltd, Surya Vidyut Ltd, Sunshakti Solar Power Projects Pvt Ltd, Torrent Saurya Urja series</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>100% (Torrent Saurya Urja 2 confirmed; others not confirmed %)</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Solar power project SPVs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>[FULL list — ~35 subsidiaries reported]</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: only a partial list could be corroborated; pull the complete AOC-1 statement from torrentpower.com/index.php/site/info/subsidiaries or the Annual Report.</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>19613.61</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10175.29</v>
+      </c>
+      <c r="D5" t="n">
+        <v>36205.82</v>
+      </c>
+      <c r="E5" t="n">
+        <v>50014.16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>19739.07</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9876.360000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>39120.52</v>
+      </c>
+      <c r="E6" t="n">
+        <v>56107.06</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FY26</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>11635.93</v>
+      </c>
+      <c r="C7" t="n">
+        <v>15027.82</v>
+      </c>
+      <c r="D7" t="n">
+        <v>41338.59</v>
+      </c>
+      <c r="E7" t="n">
+        <v>54240.52</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Verify group structure from FY26 AOC-1 statements (Phase 3)
Sheets 7-8 rebuilt from the audited AOC-1 annexures:
- Adani Power: all 19 Part A entities with exact holdings and FY26
  turnover/PAT; corrections - Mahan Energen is 94% (not 100%), Moxie
  Power (ex-Coastal Energen) is consolidated as a subsidiary at 49%
  equity (not a JV); Wangchhu Hydroelectric (Bhutan) is the sole
  AOC-1 Part B JV
- Tata Power: ~113 subsidiaries; TPREL verified at 88.57% (BlackRock
  consortium holds the balance), Tata Power-DDL and 4 Odisha discoms
  at 51% each with FY26 financials
- Torrent Power: ~60 subsidiaries (53 at 100%, 5 transmission SPVs at
  74%, Pipavav at 95%, DNH&DD at 51%)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -2113,12 +2113,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>94% (per FY26 AOC-1 — earlier reported as 100%)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>1,200 MW (2x600) coal thermal plant, MP; ex-Essar Power MP, acquired via CIRP Mar 2022.</t>
+          <t>1,200+ MW coal thermal, MP; ex-Essar Power MP (CIRP, Mar 2022). FY26: turnover ₹3,614cr, PAT ₹784cr.</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Korba Power Ltd (KPL)</t>
+          <t>Korba Power Ltd (KPL, ex-Lanco Amarkantak)</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>600 MW (2x300) coal thermal plant, Chhattisgarh; ex-Lanco Amarkantak, NCLT-approved Aug 2024.</t>
+          <t>600 MW coal thermal, Chhattisgarh (CIRP, Sep 2024). FY26: turnover ₹1,552cr, PAT ₹354cr.</t>
         </is>
       </c>
     </row>
@@ -2152,17 +2152,17 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Kutchh Power Generation Ltd (KPGL)</t>
+          <t>Moxie Power Generation Ltd (ex-Coastal Energen)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>100% (step-down, via APDL)</t>
+          <t>49% — but consolidated as a SUBSIDIARY in AOC-1 Part A (control basis), not a JV</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Held via Adani Power Dahanu Ltd (APDL); generation asset in Gujarat.</t>
+          <t>1,200 MW, Thoothukudi, Tamil Nadu. FY26: turnover ₹2,985cr, PAT ₹268cr. Listed in AOC-1 subsidiaries despite 49% equity — control established via arrangement with DAIT.</t>
         </is>
       </c>
     </row>
@@ -2174,17 +2174,17 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Adani Power Dahanu Ltd (APDL)</t>
+          <t>Vidarbha Industries Power Ltd (VIPL)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100% (acquired 07-Jul-2025)</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Holding vehicle for Dahanu-related generation assets.</t>
+          <t>600 MW, Nagpur (CIRP). FY26: turnover ₹1,327cr, PAT ₹347cr.</t>
         </is>
       </c>
     </row>
@@ -2196,17 +2196,17 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Adani Atomic Energy Ltd (AAEL)</t>
+          <t>Adani Power Dahej Ltd / Pench Thermal Energy (MP) Ltd / Kutchh Power Generation Ltd</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>100% (incorporated Feb 2026)</t>
+          <t>100% each</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>New entry into nuclear power generation, post the SHANTI Act 2025 opening the sector to private players.</t>
+          <t>Greenfield thermal project SPVs (Dahej, Pench, Kutchh).</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2218,17 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Progressive-UP Atomic Energy / Coastal-Maha Atomic Energy Ltd (CMAEL)</t>
+          <t>Anuppur Thermal Energy (MP) / Mirzapur Thermal Energy (UP) / Orrisa Thermal Energy</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>100% (step-down, incorporated 2026)</t>
+          <t>100% each (acquired/renamed 2024)</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Further nuclear-energy project SPVs.</t>
+          <t>New thermal project SPVs for capacity expansion (Anuppur, Mirzapur, Odisha sites).</t>
         </is>
       </c>
     </row>
@@ -2240,17 +2240,17 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>[6 amalgamated cos: Adani Power Maharashtra, Adani Power Rajasthan, Udupi Power Corp, Raipur Energen, Raigarh Energy Generation, Adani Power (Mundra)]</t>
+          <t>Mahan Fuel Management / Resurgent Fuel Management Ltd</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>N/A — merged into parent 1-Oct-2021</t>
+          <t>100% each</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Corporate simplification: these erstwhile subsidiaries were amalgamated directly into Adani Power Ltd.</t>
+          <t>Fuel sourcing/management SPVs.</t>
         </is>
       </c>
     </row>
@@ -2262,105 +2262,105 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>[FULL AOC-1 list]</t>
+          <t>Alcedo / Chandenvalle / Emberiza Infra Park Ltd</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: complete statutory subsidiary list with exact % holdings should be pulled from the AOC-1 annexure of the FY23/FY24 Annual Report (BSE corporate filings).</t>
+          <t>100% each</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Infrastructure park SPVs.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Tata Power Renewable Energy Ltd (TPREL)</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>~100% (verify current %)</t>
+          <t>Adani Atomic Energy Ltd (AAEL)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>100% (incorporated 11-Feb-2026)</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Renewable energy arm — utility-scale + rooftop solar and wind generation/EPC; itself has 70 subsidiaries (47 wholly-owned) as of Mar-2024.</t>
+          <t>Nuclear power entry post SHANTI Act 2025.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Tata Power Solar Systems Ltd (TPSSL)</t>
+          <t>Adani Power Middle East Ltd (AED) / Adani Power Global Pte Ltd (US$)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Verify %</t>
+          <t>100% each (incorporated 2024)</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Solar cell/module manufacturing and EPC.</t>
+          <t>Overseas ventures (Middle East; Singapore trading/holding).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Tata Power Delhi Distribution Ltd (Tata Power-DDL)</t>
+          <t>Adani Power Resources Ltd</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>51% (JV with Delhi Govt / Delhi Power Co Ltd, 49%)</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Electricity distribution licensee for North Delhi.</t>
+          <t>Resource-related SPV (immaterial size).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Adani Power</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>TP Northern/Central/Western/Southern Odisha Distribution Ltds (TPNODL/TPCODL/TPWODL/TPSODL)</t>
+          <t>[TOTAL: 19 entities in FY26 AOC-1 Part A — fully verified]</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>51% each</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Four Odisha discoms acquired 2020-21 (PPP with Odisha Govt); serve 12.6mn+ customers.</t>
+          <t>The 6 operating cos (Adani Power Maharashtra/Rajasthan, Udupi, Raipur/Raigarh Energen, Adani Power (Mundra)) were amalgamated INTO the parent effective 1-Oct-2021 and no longer appear.</t>
         </is>
       </c>
     </row>
@@ -2372,17 +2372,17 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Resurgent Power Ventures Pte Ltd (incl. NRSS XXXVI Transmission Ltd, South East UP Power Transmission Co Ltd)</t>
+          <t>Tata Power Renewable Energy Ltd (TPREL)</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Verify %</t>
+          <t>88.57% (per FY26 AOC-1 — VERIFIED; not ~100% as earlier assumed)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Acquisition vehicle for transmission-project SPVs (acquired 2023).</t>
+          <t>Renewables arm (solar/wind/rooftop/EV charging). FY26: turnover ₹11,748cr, PAT ₹1,268cr. ~11.4% held by BlackRock-led consortium since FY23 equity raise.</t>
         </is>
       </c>
     </row>
@@ -2394,17 +2394,17 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Coastal Gujarat Power Ltd (CGPL) — NOTE</t>
+          <t>Tata Power Delhi Distribution Ltd (Tata Power-DDL)</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Merged into parent, 1-Apr-2020</t>
+          <t>51% (VERIFIED per FY26 AOC-1)</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Owner/operator of Mundra UMPP; NCLT-approved merger means it is NO LONGER a separate subsidiary — Mundra is now a direct Generation-segment asset.</t>
+          <t>North Delhi discom (JV with Delhi Govt). FY26: turnover ₹10,426cr, PAT ₹1,299cr.</t>
         </is>
       </c>
     </row>
@@ -2416,83 +2416,83 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>[FULL subsidiary/JV/associate list]</t>
+          <t>TP Central / Western / Southern / Northern Odisha Distribution Ltds</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: Tata Power's 'Subsidiaries, JVs and Associates' annexure (dozens of generation/transmission/renewable SPVs) — pull from the Integrated Annual Report or AOC-1.</t>
+          <t>51% each (VERIFIED)</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Four Odisha discoms (PPP, 2020-21). FY26 turnover: TPCODL ₹6,313cr, TPWODL ₹6,355cr, TPSODL ₹2,542cr, TPNODL ₹4,769cr; all PAT-positive.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Torrent Power</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Torrent Power Grid Ltd</t>
+          <t>Tata Power Solar Systems Ltd (TPSSL)</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>74% (JV; PowerGrid Corp of India holds 26%)</t>
+          <t>In AOC-1 (100%, via TPREL structure)</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Interstate power transmission.</t>
+          <t>Solar cell/module manufacturing + EPC.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Torrent Power</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Torrent Pipavav Generation Ltd</t>
+          <t>Coastal Gujarat Power Ltd (CGPL) — NOTE</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>95%</t>
+          <t>Merged into parent, 1-Apr-2020</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Power generation, Pipavav.</t>
+          <t>Mundra UMPP is now a direct Generation-segment asset, not a subsidiary.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Torrent Power</t>
+          <t>Tata Power</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Torrent Solargen Ltd</t>
+          <t>[TOTAL: ~113 entities in FY26 AOC-1 Part A]</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Solar power generation.</t>
+          <t>Includes dozens of renewable/transmission SPVs under TPREL and Resurgent Power Ventures; full list in FY26 Annual Report pg. 666+ (AOC-1).</t>
         </is>
       </c>
     </row>
@@ -2504,17 +2504,17 @@
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Jodhpur Wind Farms Pvt Ltd</t>
+          <t>Torrent Power Grid Ltd</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>74% (VERIFIED; PowerGrid Corp holds 26%)</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Wind power generation, Rajasthan.</t>
+          <t>Interstate power transmission JV-structured subsidiary.</t>
         </is>
       </c>
     </row>
@@ -2526,17 +2526,17 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Latur Renewable Pvt Ltd</t>
+          <t>Transmission SPVs (Solapur Transmission Ltd &amp; 4 others at 74%)</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>74% each (per FY26 AOC-1)</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Renewable power generation.</t>
+          <t>Intra/interstate transmission project SPVs.</t>
         </is>
       </c>
     </row>
@@ -2548,17 +2548,17 @@
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Torrent Electricals Pvt Ltd (ex-TCL Cables Pvt Ltd)</t>
+          <t>Torrent Pipavav Generation Ltd</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>95% (VERIFIED)</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Cables/electricals manufacturing.</t>
+          <t>Power generation project, Pipavav.</t>
         </is>
       </c>
     </row>
@@ -2575,12 +2575,12 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>51% (VERIFIED)</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Power distribution licensee (DNH&amp;DD), acquired 2022.</t>
+          <t>UT power distribution licensee (acquired Apr 2022).</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2597,12 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>100% (acquired Jun 2025)</t>
+          <t>100% (acquired Jun 2026)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>2x700 MW coal-based supercritical thermal plant, Punjab.</t>
+          <t>2x700 MW supercritical coal plant, Punjab (from L&amp;T).</t>
         </is>
       </c>
     </row>
@@ -2614,17 +2614,17 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Visual Percept Solar Projects Pvt Ltd, Surya Vidyut Ltd, Sunshakti Solar Power Projects Pvt Ltd, Torrent Saurya Urja series</t>
+          <t>Torrent Solargen, Latur Renewable, Surya Vidyut, Torrent Akshay Urja, Jodhpur Wind Farms, MSKVY solar SPVs, Torrent Electricals, Newzone India, etc.</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>100% (Torrent Saurya Urja 2 confirmed; others not confirmed %)</t>
+          <t>100% each</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Solar power project SPVs.</t>
+          <t>Renewable generation SPVs (solar/wind incl. Maharashtra MSKVY series), cables/electricals, and other ventures.</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>[FULL list — ~35 subsidiaries reported]</t>
+          <t>[TOTAL: ~60 entities in FY26 AOC-1 — 53 at 100%, 5 at 74%, 1 at 95%, 1 at 51%]</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -2644,9 +2644,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: only a partial list could be corroborated; pull the complete AOC-1 statement from torrentpower.com/index.php/site/info/subsidiaries or the Annual Report.</t>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Verified from the FY26 Annual Report AOC-1 statement.</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2715,17 +2715,17 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Moxie Power Generation Ltd (ex-Coastal Energen, 1,200 MW, Tamil Nadu)</t>
+          <t>Wangchhu Hydroelectric Power Ltd (Bhutan)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>49% (JV with Dickey Alternative Investment Trust, 51%)</t>
+          <t>JV (per FY26 AOC-1 Part B — the Group's only listed associate/JV)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Adani does NOT hold majority — classified as JV/associate, not a subsidiary.</t>
+          <t>570 MW Wangchhu hydro project JV with Druk Green Power Corp (~₹6,000 cr); Shareholders Agreement Sep 2025; 'yet to commence operations' per AOC-1. VERIFIED.</t>
         </is>
       </c>
     </row>
@@ -2737,17 +2737,17 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Jaiprakash Power Ventures Ltd (JPVL)</t>
+          <t>Moxie Power Generation Ltd — RECLASSIFIED</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>24% (indirect, via resolution plan)</t>
+          <t>49% equity but consolidated as SUBSIDIARY (see Sheet 7)</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Adani Power named 'Implementing Entity'; NCLT-approved ~Mar 2026 (~₹14,535 cr resolution plan).</t>
+          <t>CORRECTION: earlier flagged as a JV; the FY26 AOC-1 lists it under Part A (Subsidiaries) — Adani has control despite 49% equity.</t>
         </is>
       </c>
     </row>
@@ -2759,17 +2759,17 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Adani Power–Druk Green Power Corp JV (Bhutan)</t>
+          <t>Jaiprakash Power Ventures Ltd (JPVL)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Not disclosed</t>
+          <t>24% (indirect, via resolution plan)</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>570 MW Wangchhu hydro project (~₹6,000 cr); Shareholders Agreement signed Sep 2025; part of a broader 5,000 MW MoU (May 2025).</t>
+          <t>Adani Power as 'Implementing Entity'; NCLT-approved ~Mar 2026 (~₹14,535 cr). Not yet in FY26 AOC-1 Part B (transaction completing post year-end).</t>
         </is>
       </c>
     </row>
@@ -2781,17 +2781,17 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Tata Power Delhi Distribution Ltd</t>
+          <t>Tata Projects, Resurgent Power Ventures (26%), industrial JVs &amp; associates</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>51% (see Sheet 7 — sometimes classified as JV given 49% Delhi Govt partner)</t>
+          <t>Various</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Listed here for completeness; treated as subsidiary in Sheet 7 given majority control.</t>
+          <t>Tata Power holds numerous associates/JVs (share of profit ₹708cr FY26, ₹793cr FY25 per consolidated P&amp;L); full Part B list in FY26 Annual Report AOC-1.</t>
         </is>
       </c>
     </row>
@@ -2808,56 +2808,34 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Stake not disclosed</t>
+          <t>Stake not disclosed in extract</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>1,125 MW hydro project under development.</t>
+          <t>1,125 MW hydro project under development with Druk Green.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Tata Power</t>
+          <t>Torrent Power</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>[Other associates/JVs]</t>
+          <t>Associates (2 per earlier AOC-1 references)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: Tata Power's full associates/JV list not retrievable via search — pull from Annual Report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Torrent Power</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>2 associate companies (per AOC-1 reference)</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Not disclosed</t>
-        </is>
-      </c>
-      <c r="D12" s="18" t="inlineStr">
-        <is>
-          <t>VERIFY: names/business of the 2 associate companies not found via search — pull from Annual Report AOC-1.</t>
+          <t>Not extracted</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Torrent's FY26 AOC-1 Part B not extracted in this pass — the Part A subsidiary data above is verified; pull Part B from the same annexure if associate detail is needed.</t>
         </is>
       </c>
     </row>
@@ -4525,7 +4503,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>7. Complete subsidiary/associate/JV lists with exact % holdings — pull the AOC-1 annexure from each company's Annual Report (now in the repo — worth a follow-up extraction pass).</t>
+          <t>7. Subsidiary lists — DONE: Sheets 7-8 now carry the verified FY26 AOC-1 data (Adani 19 entities incl. Mahan at 94% and Moxie consolidated at 49%; Tata ~113 entities incl. TPREL at 88.57%; Torrent ~60 entities). Only Torrent's associates (Part B) remain unextracted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verify investments (ex-subs/associates/JVs) from FY23 notes (Phase 4)
Sheet 9 now carries figures extracted from the consolidated Investments
notes of the three FY2022-23 Annual Reports:
- Adani Power: non-current ₹42.51cr (OCCDs of Sal Technologies ₹42.50cr,
  NSC, negligible FVTOCI equity) + current MFs ₹611.54cr (SBI Liquid/
  Overnight), up from ₹183.24cr FY22
- Tata Power: ₹1,301.21cr non-current third-party portfolio incl.
  ₹128.10cr government securities - replaces the earlier unverified
  ~₹12,064cr figure which conflated associate/JV carrying values
- Torrent Power: GERC-mandated GoI contingency-reserve bonds ~₹15.94cr
  + current investments ₹682.31cr (mostly MFs)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -2896,14 +2896,14 @@
           <t>Adani Power</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>No disclosed breakdown of non-subsidiary investment portfolio (govt securities, mutual funds, bonds) found for FY19-FY23. This sits in the balance-sheet 'Investments' / 'Other Financial Assets' note.</t>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>VERIFIED from FY23 consolidated Investments notes: NON-CURRENT — ₹42.51cr total as at 31-Mar-2023 (vs ₹0.01cr FY22), comprising ₹42.50cr of 0.001% Optionally Convertible Cumulative Debentures of Sal Technologies and Solutions Ltd (4.25cr units, new in FY23), a ₹0.01cr National Saving Certificate, and a negligible FVTOCI equity stake in Adani Naval Defence Systems &amp; Technologies Ltd. CURRENT — ₹611.54cr in unquoted mutual funds (SBI Liquid Fund ₹608.42cr + SBI Overnight Fund ₹3.12cr) vs ₹183.24cr (FY22, SBI Overnight only). Pattern: treasury parked in liquid MFs, scale rising with cash generation; almost no discretionary long-term securities portfolio.</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>GAP — pull from Annual Report</t>
+          <t>VERIFIED (FY23 Annual Report)</t>
         </is>
       </c>
     </row>
@@ -2913,14 +2913,14 @@
           <t>Tata Power</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>One unverified secondary snippet suggested non-current investments of ~₹12,064.55 crore as of March 2023 (consolidation basis unclear, source of uncertain provenance).</t>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>VERIFIED from FY23 consolidated Investments note: non-current investments OTHER than associates/JVs totalled ₹1,301.21cr as at 31-Mar-2023 (vs ₹1,169.81cr FY22), comprising equity shares carried at FVTOCI/FVTPL and Government Securities (unquoted) of ₹128.10cr (FY22: ₹124.26cr). The earlier secondary-source figure of '~₹12,064cr non-current investments' conflated investments in associates/JVs (equity-method carrying values) with this third-party portfolio — use ₹1,301cr for the ex-subsidiary/associate/JV basis the assignment asks for.</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>UNVERIFIED — do not cite without checking the FY23 balance sheet directly</t>
+          <t>VERIFIED (FY23 Annual Report) — replaces earlier unverified figure</t>
         </is>
       </c>
     </row>
@@ -2930,21 +2930,21 @@
           <t>Torrent Power</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Holds Government of India Bonds as part of a regulatory 'contingency reserve' required under GERC Multi-Year Tariff Regulations (tied to its Gujarat distribution license) — i.e., regulatory-mandated, not discretionary treasury investment. No itemized schedule found.</t>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>VERIFIED from FY23 consolidated Investments notes: NON-CURRENT — quoted investments (incl. Government of India bonds held as the GERC Multi-Year-Tariff-mandated 'contingency reserve' for its Gujarat distribution licences) of ~₹15.94cr market value ₹15.70cr as at 31-Mar-2023 (down from ₹132.82cr FY22 as bonds matured/were reclassified). CURRENT — ₹682.31cr total (vs ₹253.27cr FY22): unquoted mutual funds ₹656.03cr + statutory contingency-reserve investments ₹1.93cr + other ₹24.35cr. The GoI-bond holdings are regulatory-mandated (usable only for GERC-specified purposes), not discretionary treasury.</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>PARTIAL — nature identified, amounts not found</t>
+          <t>VERIFIED (FY23 Annual Report)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>Note: this section requires the 'Investments' note from each company's FY2023 standalone/consolidated Balance Sheet — none of the three companies' figures could be reliably retrieved via web search in this session.</t>
+          <t>All three companies' figures above are now extracted directly from the consolidated 'Investments' notes of the FY2022-23 Annual Reports uploaded to the repo. Common pattern: all three park treasury cash in liquid/overnight mutual funds; Torrent additionally holds regulatory-mandated GoI bonds (GERC contingency reserve); none runs a material discretionary securities portfolio.</t>
         </is>
       </c>
     </row>
@@ -4510,7 +4510,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>8. Investments note (ex subsidiaries/associates/JVs) as at 31-Mar-2023 — pull from each company's Balance Sheet notes.</t>
+          <t>8. Investments (ex subsidiaries/associates/JVs) as at 31-Mar-2023 — DONE: Sheet 9 now carries verified figures from all three FY23 Annual Reports (Adani ₹42.51cr non-current + ₹611.54cr MFs; Tata ₹1,301.21cr; Torrent ₹15.94cr bonds + ₹682.31cr current).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Sheet 11 with Nifty 50 market-index data (Phase 5 final)
Parsed the corrected NIFTY50_weeklyreal.htm (54 weekly closes): market
returned -3.6% over the year, 12.3% annualized volatility.

Sheet 11 now fully computed with no pending cells:
- Market betas vs Nifty 50: Adani 1.13, Tata 0.62, Torrent 1.46
- All three stocks beat the market (Adani by ~88 points)
- Nifty 50 series added to Weekly_Price_Data and stats table

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -36,7 +36,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +96,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00008000"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00C00000"/>
     </font>
   </fonts>
@@ -143,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,6 +180,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3438,7 +3443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3522,9 +3527,9 @@
           <t>36,231.65</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>24,968.40</t>
         </is>
       </c>
     </row>
@@ -3554,9 +3559,9 @@
           <t>39,381.25</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>24,078.50</t>
         </is>
       </c>
     </row>
@@ -3586,9 +3591,9 @@
           <t>33,098.30 - 40,878.00</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>22,713.10 - 26,328.55</t>
         </is>
       </c>
     </row>
@@ -3618,9 +3623,9 @@
           <t>+8.7%</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>-3.6%</t>
         </is>
       </c>
     </row>
@@ -3650,9 +3655,9 @@
           <t>2.30%</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>1.70%</t>
         </is>
       </c>
     </row>
@@ -3682,119 +3687,183 @@
           <t>16.6%</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>12.3%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Beta vs Nifty Energy (COMPUTED)</t>
+          <t>Beta vs Nifty 50 / market (COMPUTED)</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
+          <t>0.62</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
           <t>0.03</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>1.00</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
+          <t>Beta vs Nifty Energy / sector (COMPUTED)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Return vs market (stock - Nifty 50)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>+87.7 pts</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>-2.5 pts</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>+10.3 pts</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>+12.3 pts</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
           <t>Return vs sector (stock - Nifty Energy)</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>+75.4 pts</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>-14.7 pts</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>-1.9 pts</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>Nifty 50 note</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>The NIFTY50_weekly.htm file saved to the repo was the ^NSEI Charts/summary page, not the Historical Data page, so it contains no weekly table. To complete the market-index column: open finance.yahoo.com/quote/%5ENSEI/history/?frequency=1wk, scroll to load all rows, Ctrl+S as HTML, and replace NIFTY50_weekly.htm in the repo. Everything else on this sheet is final, computed from real data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Data note</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>COMPLETE: all five series (3 stocks + Nifty 50 + Nifty Energy) parsed from the Yahoo Finance Historical Data pages saved in the repo (54 weekly adjusted-close points each, 14-Jul-2025 to 15-Jul-2026, split-adjusted). Weekly returns, standard deviations, annualized volatility, and betas computed from this data - see the Weekly_Price_Data sheet for the full series and the rebased performance chart below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Comments — which share is most volatile?</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="130" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>ANSWER (computed from 54 weekly observations, split-adjusted): ADANI POWER is the most volatile of the three — weekly-return standard deviation 4.95% (annualized ~36%), vs Torrent Power 4.55% (~33%) and Tata Power 2.90% (~21%). The sector index (Nifty Energy) sat at 2.30% weekly (~17% annualized) — all three stocks were roughly 1.3-2.2x as volatile as their sector index. RETURNS: Adani Power massively outperformed (+84% vs the sector's +9%), Torrent Power roughly tracked the sector (+6.8%), and Tata Power underperformed (-6.0%). Note the LOW computed betas vs Nifty Energy (0.03-0.54): Nifty Energy is dominated by Reliance/ONGC (oil &amp; gas), so these power stocks move on company-specific news far more than on the 'sector' index — high volatility with low index correlation. Interpret beta accordingly, and recompute vs Nifty 50 once the market-index file is added for the conventional market beta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
+    <row r="23" ht="130" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>ANSWER (computed from 54 weekly observations, split-adjusted): ADANI POWER is the most volatile of the three — weekly-return standard deviation 4.95% (annualized ~36%), vs Torrent Power 4.55% (~33%) and Tata Power 2.90% (~21%). The sector index (Nifty Energy) sat at 2.30% weekly (~17% annualized) — all three stocks were roughly 1.3-2.2x as volatile as their sector index. RETURNS: Adani Power massively outperformed (+84% vs the sector's +9%), Torrent Power roughly tracked the sector (+6.8%), and Tata Power underperformed (-6.0%). Note the LOW computed betas vs Nifty Energy (0.03-0.54): Nifty Energy is dominated by Reliance/ONGC (oil &amp; gas), so these power stocks move on company-specific news far more than on the 'sector' index — high volatility with low index correlation. Interpret beta accordingly. VS THE MARKET: Nifty 50 fell -3.6% over the window, so all three power stocks outperformed the broad market (Adani by ~88 points); market betas vs Nifty 50 are 1.13 (Adani), 0.62 (Tata) and 1.46 (Torrent).</t>
+        </is>
+      </c>
+    </row>
     <row r="24"/>
     <row r="25"/>
     <row r="26"/>
     <row r="27"/>
     <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A16:F18"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A18:F20"/>
+    <mergeCell ref="A23:F30"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A21:F28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3854,7 +3923,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Nifty 50 (PENDING)</t>
+          <t>Nifty 50</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -3916,6 +3985,9 @@
       <c r="E2" t="n">
         <v>36231.65</v>
       </c>
+      <c r="F2" t="n">
+        <v>24968.4</v>
+      </c>
       <c r="K2" t="n">
         <v>100</v>
       </c>
@@ -3947,6 +4019,9 @@
       <c r="E3" t="n">
         <v>35250.5</v>
       </c>
+      <c r="F3" t="n">
+        <v>24837</v>
+      </c>
       <c r="G3" t="n">
         <v>-0.041453</v>
       </c>
@@ -3990,6 +4065,9 @@
       <c r="E4" t="n">
         <v>34889</v>
       </c>
+      <c r="F4" t="n">
+        <v>24565.35</v>
+      </c>
       <c r="G4" t="n">
         <v>-0.005263</v>
       </c>
@@ -4033,6 +4111,9 @@
       <c r="E5" t="n">
         <v>34391.95</v>
       </c>
+      <c r="F5" t="n">
+        <v>24363.3</v>
+      </c>
       <c r="G5" t="n">
         <v>0.01746</v>
       </c>
@@ -4076,6 +4157,9 @@
       <c r="E6" t="n">
         <v>34469.05</v>
       </c>
+      <c r="F6" t="n">
+        <v>24631.3</v>
+      </c>
       <c r="G6" t="n">
         <v>0.012394</v>
       </c>
@@ -4119,6 +4203,9 @@
       <c r="E7" t="n">
         <v>34507.6</v>
       </c>
+      <c r="F7" t="n">
+        <v>24870.1</v>
+      </c>
       <c r="G7" t="n">
         <v>0.01755</v>
       </c>
@@ -4162,6 +4249,9 @@
       <c r="E8" t="n">
         <v>33638.65</v>
       </c>
+      <c r="F8" t="n">
+        <v>24426.85</v>
+      </c>
       <c r="G8" t="n">
         <v>0.010685</v>
       </c>
@@ -4205,6 +4295,9 @@
       <c r="E9" t="n">
         <v>34297.9</v>
       </c>
+      <c r="F9" t="n">
+        <v>24741</v>
+      </c>
       <c r="G9" t="n">
         <v>0.015067</v>
       </c>
@@ -4248,6 +4341,9 @@
       <c r="E10" t="n">
         <v>34940.3</v>
       </c>
+      <c r="F10" t="n">
+        <v>25114</v>
+      </c>
       <c r="G10" t="n">
         <v>0.06372</v>
       </c>
@@ -4291,6 +4387,9 @@
       <c r="E11" t="n">
         <v>35745.75</v>
       </c>
+      <c r="F11" t="n">
+        <v>25327.05</v>
+      </c>
       <c r="G11" t="n">
         <v>0.09382500000000001</v>
       </c>
@@ -4334,6 +4433,9 @@
       <c r="E12" t="n">
         <v>34830</v>
       </c>
+      <c r="F12" t="n">
+        <v>24654.7</v>
+      </c>
       <c r="G12" t="n">
         <v>0.030801</v>
       </c>
@@ -4377,6 +4479,9 @@
       <c r="E13" t="n">
         <v>35375.9</v>
       </c>
+      <c r="F13" t="n">
+        <v>24894.25</v>
+      </c>
       <c r="G13" t="n">
         <v>0.007726</v>
       </c>
@@ -4420,6 +4525,9 @@
       <c r="E14" t="n">
         <v>35393.95</v>
       </c>
+      <c r="F14" t="n">
+        <v>25285.35</v>
+      </c>
       <c r="G14" t="n">
         <v>0.015742</v>
       </c>
@@ -4463,6 +4571,9 @@
       <c r="E15" t="n">
         <v>35395.7</v>
       </c>
+      <c r="F15" t="n">
+        <v>25709.85</v>
+      </c>
       <c r="G15" t="n">
         <v>0.108751</v>
       </c>
@@ -4506,6 +4617,9 @@
       <c r="E16" t="n">
         <v>35626.9</v>
       </c>
+      <c r="F16" t="n">
+        <v>25795.15</v>
+      </c>
       <c r="G16" t="n">
         <v>0.010483</v>
       </c>
@@ -4549,6 +4663,9 @@
       <c r="E17" t="n">
         <v>36275.95</v>
       </c>
+      <c r="F17" t="n">
+        <v>25722.1</v>
+      </c>
       <c r="G17" t="n">
         <v>-0.058848</v>
       </c>
@@ -4592,6 +4709,9 @@
       <c r="E18" t="n">
         <v>35790.3</v>
       </c>
+      <c r="F18" t="n">
+        <v>25492.3</v>
+      </c>
       <c r="G18" t="n">
         <v>-0.040355</v>
       </c>
@@ -4635,6 +4755,9 @@
       <c r="E19" t="n">
         <v>36261.1</v>
       </c>
+      <c r="F19" t="n">
+        <v>25910.05</v>
+      </c>
       <c r="G19" t="n">
         <v>0.016042</v>
       </c>
@@ -4678,6 +4801,9 @@
       <c r="E20" t="n">
         <v>35852.4</v>
       </c>
+      <c r="F20" t="n">
+        <v>26068.15</v>
+      </c>
       <c r="G20" t="n">
         <v>-0.031122</v>
       </c>
@@ -4721,6 +4847,9 @@
       <c r="E21" t="n">
         <v>35548.3</v>
       </c>
+      <c r="F21" t="n">
+        <v>26202.95</v>
+      </c>
       <c r="G21" t="n">
         <v>-0.010931</v>
       </c>
@@ -4764,6 +4893,9 @@
       <c r="E22" t="n">
         <v>34971.8</v>
       </c>
+      <c r="F22" t="n">
+        <v>26186.45</v>
+      </c>
       <c r="G22" t="n">
         <v>-0.025154</v>
       </c>
@@ -4807,6 +4939,9 @@
       <c r="E23" t="n">
         <v>35039.85</v>
       </c>
+      <c r="F23" t="n">
+        <v>26046.95</v>
+      </c>
       <c r="G23" t="n">
         <v>0.004938</v>
       </c>
@@ -4850,6 +4985,9 @@
       <c r="E24" t="n">
         <v>34796.4</v>
       </c>
+      <c r="F24" t="n">
+        <v>25966.4</v>
+      </c>
       <c r="G24" t="n">
         <v>-0.018894</v>
       </c>
@@ -4893,6 +5031,9 @@
       <c r="E25" t="n">
         <v>35058.8</v>
       </c>
+      <c r="F25" t="n">
+        <v>26042.3</v>
+      </c>
       <c r="G25" t="n">
         <v>0.003033</v>
       </c>
@@ -4936,6 +5077,9 @@
       <c r="E26" t="n">
         <v>36275.65</v>
       </c>
+      <c r="F26" t="n">
+        <v>26328.55</v>
+      </c>
       <c r="G26" t="n">
         <v>0.042056</v>
       </c>
@@ -4979,6 +5123,9 @@
       <c r="E27" t="n">
         <v>34409.3</v>
       </c>
+      <c r="F27" t="n">
+        <v>25683.3</v>
+      </c>
       <c r="G27" t="n">
         <v>-0.043801</v>
       </c>
@@ -5022,6 +5169,9 @@
       <c r="E28" t="n">
         <v>34346.35</v>
       </c>
+      <c r="F28" t="n">
+        <v>25694.35</v>
+      </c>
       <c r="G28" t="n">
         <v>0.006705</v>
       </c>
@@ -5065,6 +5215,9 @@
       <c r="E29" t="n">
         <v>33098.3</v>
       </c>
+      <c r="F29" t="n">
+        <v>25048.65</v>
+      </c>
       <c r="G29" t="n">
         <v>-0.067798</v>
       </c>
@@ -5108,6 +5261,9 @@
       <c r="E30" t="n">
         <v>35138.05</v>
       </c>
+      <c r="F30" t="n">
+        <v>24825.45</v>
+      </c>
       <c r="G30" t="n">
         <v>-0.000827</v>
       </c>
@@ -5151,6 +5307,9 @@
       <c r="E31" t="n">
         <v>36451.7</v>
       </c>
+      <c r="F31" t="n">
+        <v>25693.7</v>
+      </c>
       <c r="G31" t="n">
         <v>0.149718</v>
       </c>
@@ -5194,6 +5353,9 @@
       <c r="E32" t="n">
         <v>35709.9</v>
       </c>
+      <c r="F32" t="n">
+        <v>25471.1</v>
+      </c>
       <c r="G32" t="n">
         <v>-0.084064</v>
       </c>
@@ -5237,6 +5399,9 @@
       <c r="E33" t="n">
         <v>36581.15</v>
       </c>
+      <c r="F33" t="n">
+        <v>25571.25</v>
+      </c>
       <c r="G33" t="n">
         <v>0.020014</v>
       </c>
@@ -5280,6 +5445,9 @@
       <c r="E34" t="n">
         <v>37045.2</v>
       </c>
+      <c r="F34" t="n">
+        <v>25178.65</v>
+      </c>
       <c r="G34" t="n">
         <v>-0.01815</v>
       </c>
@@ -5323,6 +5491,9 @@
       <c r="E35" t="n">
         <v>36319.6</v>
       </c>
+      <c r="F35" t="n">
+        <v>24450.45</v>
+      </c>
       <c r="G35" t="n">
         <v>-0.007993999999999999</v>
       </c>
@@ -5366,6 +5537,9 @@
       <c r="E36" t="n">
         <v>36071.85</v>
       </c>
+      <c r="F36" t="n">
+        <v>23151.1</v>
+      </c>
       <c r="G36" t="n">
         <v>0.054536</v>
       </c>
@@ -5409,6 +5583,9 @@
       <c r="E37" t="n">
         <v>35908.3</v>
       </c>
+      <c r="F37" t="n">
+        <v>23114.5</v>
+      </c>
       <c r="G37" t="n">
         <v>0.033909</v>
       </c>
@@ -5452,6 +5629,9 @@
       <c r="E38" t="n">
         <v>35214.8</v>
       </c>
+      <c r="F38" t="n">
+        <v>22819.6</v>
+      </c>
       <c r="G38" t="n">
         <v>0.015705</v>
       </c>
@@ -5495,6 +5675,9 @@
       <c r="E39" t="n">
         <v>35299.4</v>
       </c>
+      <c r="F39" t="n">
+        <v>22713.1</v>
+      </c>
       <c r="G39" t="n">
         <v>0.039306</v>
       </c>
@@ -5538,6 +5721,9 @@
       <c r="E40" t="n">
         <v>37174.6</v>
       </c>
+      <c r="F40" t="n">
+        <v>24050.6</v>
+      </c>
       <c r="G40" t="n">
         <v>0.099019</v>
       </c>
@@ -5581,6 +5767,9 @@
       <c r="E41" t="n">
         <v>38881.75</v>
       </c>
+      <c r="F41" t="n">
+        <v>24353.55</v>
+      </c>
       <c r="G41" t="n">
         <v>0.12906</v>
       </c>
@@ -5624,6 +5813,9 @@
       <c r="E42" t="n">
         <v>39903.75</v>
       </c>
+      <c r="F42" t="n">
+        <v>23897.95</v>
+      </c>
       <c r="G42" t="n">
         <v>0.072544</v>
       </c>
@@ -5667,6 +5859,9 @@
       <c r="E43" t="n">
         <v>40771.9</v>
       </c>
+      <c r="F43" t="n">
+        <v>23997.55</v>
+      </c>
       <c r="G43" t="n">
         <v>0.042039</v>
       </c>
@@ -5710,6 +5905,9 @@
       <c r="E44" t="n">
         <v>40795.8</v>
       </c>
+      <c r="F44" t="n">
+        <v>24176.15</v>
+      </c>
       <c r="G44" t="n">
         <v>0.015686</v>
       </c>
@@ -5753,6 +5951,9 @@
       <c r="E45" t="n">
         <v>39816.85</v>
       </c>
+      <c r="F45" t="n">
+        <v>23643.5</v>
+      </c>
       <c r="G45" t="n">
         <v>-0.017752</v>
       </c>
@@ -5796,6 +5997,9 @@
       <c r="E46" t="n">
         <v>40237.6</v>
       </c>
+      <c r="F46" t="n">
+        <v>23719.3</v>
+      </c>
       <c r="G46" t="n">
         <v>-0.009081000000000001</v>
       </c>
@@ -5839,6 +6043,9 @@
       <c r="E47" t="n">
         <v>40878</v>
       </c>
+      <c r="F47" t="n">
+        <v>23547.75</v>
+      </c>
       <c r="G47" t="n">
         <v>0.109657</v>
       </c>
@@ -5882,6 +6089,9 @@
       <c r="E48" t="n">
         <v>40346.1</v>
       </c>
+      <c r="F48" t="n">
+        <v>23366.7</v>
+      </c>
       <c r="G48" t="n">
         <v>-0.044254</v>
       </c>
@@ -5925,6 +6135,9 @@
       <c r="E49" t="n">
         <v>39244.45</v>
       </c>
+      <c r="F49" t="n">
+        <v>23622.9</v>
+      </c>
       <c r="G49" t="n">
         <v>-0.040972</v>
       </c>
@@ -5968,6 +6181,9 @@
       <c r="E50" t="n">
         <v>40548.1</v>
       </c>
+      <c r="F50" t="n">
+        <v>24013.1</v>
+      </c>
       <c r="G50" t="n">
         <v>0.038956</v>
       </c>
@@ -6011,6 +6227,9 @@
       <c r="E51" t="n">
         <v>39637</v>
       </c>
+      <c r="F51" t="n">
+        <v>24056</v>
+      </c>
       <c r="G51" t="n">
         <v>-0.010744</v>
       </c>
@@ -6054,6 +6273,9 @@
       <c r="E52" t="n">
         <v>39178.6</v>
       </c>
+      <c r="F52" t="n">
+        <v>24270.85</v>
+      </c>
       <c r="G52" t="n">
         <v>-0.032625</v>
       </c>
@@ -6097,6 +6319,9 @@
       <c r="E53" t="n">
         <v>39242.05</v>
       </c>
+      <c r="F53" t="n">
+        <v>24206.9</v>
+      </c>
       <c r="G53" t="n">
         <v>-0.015059</v>
       </c>
@@ -6137,6 +6362,9 @@
       <c r="D54" t="n">
         <v>1465.3</v>
       </c>
+      <c r="F54" t="n">
+        <v>24052.05</v>
+      </c>
       <c r="G54" t="n">
         <v>0.03534</v>
       </c>
@@ -6173,6 +6401,9 @@
       </c>
       <c r="E55" t="n">
         <v>39381.25</v>
+      </c>
+      <c r="F55" t="n">
+        <v>24078.5</v>
       </c>
       <c r="G55" t="n">
         <v>-0.031834</v>
@@ -6521,7 +6752,7 @@
       <c r="D19" s="11" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>Note on this section</t>
         </is>
@@ -7285,7 +7516,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>5. Weekly price series — LARGELY DONE: 54-week adjusted-close series for all 3 stocks + Nifty Energy parsed from Yahoo HTML files in the repo; returns, std-dev volatility and sector betas computed in Sheet 11. Outstanding: Nifty 50 (wrong page was saved — re-save the ^NSEI Historical Data page) and year-end FY19-FY26 prices for Sheet 2.</t>
+          <t>5. Weekly price series — DONE: 54-week adjusted-close series for all 3 stocks + Nifty 50 + Nifty Energy parsed from Yahoo HTML files in the repo; returns, volatility, and market &amp; sector betas computed in Sheet 11. Still open: year-end FY19-FY26 share prices for the Sheet 2 growth table (needs older price history).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Narrow analysis window to FY22-FY26 (last five years)
Per user request, removed all FY19/FY20/FY21 data from the workbook:
- Sheet 2 growth table now runs FY22-FY26 with 4-yr CAGR; all cells
  primary-verified except FY-end share prices and two employee counts
- Sheet 3 ratios recomputed on the 5-year window
- Sheet 6 segment tables trimmed to FY22-FY26 with growth stats rebased
- Charts (revenue, PAT, assets, segments) rebuilt on FY22-FY26
- Sources & Gaps updated to the new scope

Historical event references (Odisha discom acquisitions 2020-21, Tata's
2020 preferential allotment) retained as acquisition/financing history.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -269,7 +269,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue / Total Income Trend, FY19-FY26 (₹ crore)</a:t>
+              <a:t>Revenue / Total Income Trend, FY22-FY26 (₹ crore)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -294,12 +294,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$2:$A$9</f>
+              <f>'2b_Growth_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$B$2:$B$9</f>
+              <f>'2b_Growth_Chart_Data'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -318,12 +318,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$2:$A$9</f>
+              <f>'2b_Growth_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$C$2:$C$9</f>
+              <f>'2b_Growth_Chart_Data'!$C$2:$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -342,12 +342,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$2:$A$9</f>
+              <f>'2b_Growth_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$D$2:$D$9</f>
+              <f>'2b_Growth_Chart_Data'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -429,7 +429,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Net Profit / PAT Trend, FY19-FY26 (₹ crore)</a:t>
+              <a:t>Net Profit / PAT Trend, FY22-FY26 (₹ crore)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -444,7 +444,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!B11</f>
+              <f>'2b_Growth_Chart_Data'!B8</f>
             </strRef>
           </tx>
           <spPr>
@@ -454,12 +454,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$12:$A$19</f>
+              <f>'2b_Growth_Chart_Data'!$A$9:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$B$12:$B$19</f>
+              <f>'2b_Growth_Chart_Data'!$B$9:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -468,7 +468,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!C11</f>
+              <f>'2b_Growth_Chart_Data'!C8</f>
             </strRef>
           </tx>
           <spPr>
@@ -478,12 +478,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$12:$A$19</f>
+              <f>'2b_Growth_Chart_Data'!$A$9:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$C$12:$C$19</f>
+              <f>'2b_Growth_Chart_Data'!$C$9:$C$13</f>
             </numRef>
           </val>
         </ser>
@@ -492,7 +492,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!D11</f>
+              <f>'2b_Growth_Chart_Data'!D8</f>
             </strRef>
           </tx>
           <spPr>
@@ -502,12 +502,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$12:$A$19</f>
+              <f>'2b_Growth_Chart_Data'!$A$9:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$D$12:$D$19</f>
+              <f>'2b_Growth_Chart_Data'!$D$9:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -589,7 +589,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Total Assets Trend, FY20-FY26 (₹ crore, consolidated)</a:t>
+              <a:t>Total Assets Trend, FY22-FY26 (₹ crore, consolidated)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -604,7 +604,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!B21</f>
+              <f>'2b_Growth_Chart_Data'!B15</f>
             </strRef>
           </tx>
           <spPr>
@@ -614,12 +614,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$22:$A$28</f>
+              <f>'2b_Growth_Chart_Data'!$A$16:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$B$22:$B$28</f>
+              <f>'2b_Growth_Chart_Data'!$B$16:$B$20</f>
             </numRef>
           </val>
         </ser>
@@ -628,7 +628,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!C21</f>
+              <f>'2b_Growth_Chart_Data'!C15</f>
             </strRef>
           </tx>
           <spPr>
@@ -638,12 +638,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$22:$A$28</f>
+              <f>'2b_Growth_Chart_Data'!$A$16:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$C$22:$C$28</f>
+              <f>'2b_Growth_Chart_Data'!$C$16:$C$20</f>
             </numRef>
           </val>
         </ser>
@@ -652,7 +652,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'2b_Growth_Chart_Data'!D21</f>
+              <f>'2b_Growth_Chart_Data'!D15</f>
             </strRef>
           </tx>
           <spPr>
@@ -662,12 +662,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$A$22:$A$28</f>
+              <f>'2b_Growth_Chart_Data'!$A$16:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2b_Growth_Chart_Data'!$D$22:$D$28</f>
+              <f>'2b_Growth_Chart_Data'!$D$16:$D$20</f>
             </numRef>
           </val>
         </ser>
@@ -749,7 +749,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Segment Revenue Trends FY21-FY26 (₹ crore): Tata segments vs Adani Generation</a:t>
+              <a:t>Segment Revenue Trends FY22-FY26 (₹ crore): Tata segments vs Adani Generation</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -781,12 +781,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$B$2:$B$7</f>
+              <f>'6b_Segment_Chart_Data'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$C$2:$C$7</f>
+              <f>'6b_Segment_Chart_Data'!$C$2:$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$D$2:$D$7</f>
+              <f>'6b_Segment_Chart_Data'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -877,12 +877,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$A$2:$A$7</f>
+              <f>'6b_Segment_Chart_Data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'6b_Segment_Chart_Data'!$E$2:$E$7</f>
+              <f>'6b_Segment_Chart_Data'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1304,92 +1304,17 @@
     <author>Research Agent</author>
   </authors>
   <commentList>
-    <comment ref="B9" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
         <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
       </text>
     </comment>
-    <comment ref="C10" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="E10" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="G10" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="C14" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="C15" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="C16" authorId="0" shapeId="0">
+    <comment ref="D10" authorId="0" shapeId="0">
       <text>
         <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
       </text>
     </comment>
     <comment ref="D16" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="G16" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B19" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B20" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B21" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="B22" authorId="0" shapeId="0">
-      <text>
-        <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
-      </text>
-    </comment>
-    <comment ref="C22" authorId="0" shapeId="0">
       <text>
         <t>Not independently verifiable via web search in this session — pull directly from screener.in / moneycontrol / NSE-BSE filings / the company's Annual Report before final submission.</t>
       </text>
@@ -1419,21 +1344,6 @@
         <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
       </text>
     </comment>
-    <comment ref="G26" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="H26" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="I26" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
     <comment ref="B27" authorId="0" shapeId="0">
       <text>
         <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
@@ -1459,21 +1369,6 @@
         <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
       </text>
     </comment>
-    <comment ref="G27" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="H27" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="I27" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
     <comment ref="B28" authorId="0" shapeId="0">
       <text>
         <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
@@ -1495,21 +1390,6 @@
       </text>
     </comment>
     <comment ref="F28" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="G28" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="H28" authorId="0" shapeId="0">
-      <text>
-        <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
-      </text>
-    </comment>
-    <comment ref="I28" authorId="0" shapeId="0">
       <text>
         <t>Historical FY-end (31 March) closing prices were not retrievable via search in this session. Pull directly from NSE historical data / Yahoo Finance (finance.yahoo.com/quote/&lt;TICKER&gt;.NS/history) — NOTE: Adani Power did a 1:5 stock split effective 22-Sep-2025, so use SPLIT-ADJUSTED prices for a like-for-like series.</t>
       </text>
@@ -3417,7 +3297,7 @@
     <row r="21" ht="100" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>All three companies have been actively de-leveraging and improving credit ratings over the last five years — a sector-wide trend as thermal-generation cash flows normalized post-COVID and renewable capex was increasingly funded with cheaper, longer-tenor debt. Adani Power's improvement is the most dramatic in relative terms (net debt/EBITDA from ~4x to ~1.4x within two years), consistent with its swing from losses to strong profitability. Tata Power funded its FY20 deleveraging via a promoter-only preferential allotment rather than a public offering, keeping the raise off the open market. Torrent Power is notable for having gone ~30 years without a public equity raise before its Dec-2024 QIP — a signal of a more conservative, debt/promoter-funded capital structure historically, now shifting toward institutional equity to fund its large (₹80,000 cr) five-year capex programme.</t>
+          <t>All three companies have been actively de-leveraging and improving credit ratings over the last five years — a sector-wide trend as thermal-generation cash flows normalized post-COVID and renewable capex was increasingly funded with cheaper, longer-tenor debt. Adani Power's improvement is the most dramatic in relative terms (net debt/EBITDA from ~4x to ~1.4x within two years), consistent with its swing from losses to strong profitability. Tata Power funded its 2020 deleveraging via a promoter-only preferential allotment rather than a public offering, keeping the raise off the open market. Torrent Power is notable for having gone ~30 years without a public equity raise before its Dec-2024 QIP — a signal of a more conservative, debt/promoter-funded capital structure historically, now shifting toward institutional equity to fund its large (₹80,000 cr) five-year capex programme.</t>
         </is>
       </c>
     </row>
@@ -7469,7 +7349,7 @@
     <row r="6" ht="115" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>This workbook was built using automated web search (news wires, brokerage research notes, exchange press releases, and secondary financial-data aggregators such as Trendlyne, ScanX, HDFC Sky, Business Standard, BusinessToday, Equitymaster) inside a sandboxed research session. Direct scripted/API access to the PRIMARY sources you were asked to use — screener.in, moneycontrol.com, NSE India (nseindia.com), BSE India (bseindia.com), and the companies' own Annual Report PDFs (adanipower.com, tatapower.com, torrentpower.com) — was blocked (HTTP 403) for automated fetches in this environment. All numbers not otherwise flagged therefore come from search-engine snippets of secondary coverage of those primary sources, not the primary documents themselves. UPDATE: the user subsequently uploaded the actual Integrated Annual Report PDFs covering — Adani Power FY20-21, FY22-23, FY23-24 (financials section), FY24-25 and FY25-26; Tata Power FY21-22, FY22-23, FY23-24, FY24-25 and FY25-26; Torrent Power FY20-21 through FY25-26 (all six). Using each report's current + prior-year comparative columns, the consolidated Revenue/Total Income, PAT and Total Assets series in Sheet 2 are now PRIMARY-VERIFIED for FY20-FY26 (Adani, Torrent) and FY21-FY26 (Tata), and standalone employee counts were extracted where disclosed. Only FY19 (all metrics beyond secondary-sourced revenue/PAT) and the share-price rows remain unverified/yellow. Segment tables, AOC-1 subsidiary lists and the Investments notes are IN these PDFs but not yet extracted into Sheets 6-9.</t>
+          <t>This workbook was built using automated web search (news wires, brokerage research notes, exchange press releases, and secondary financial-data aggregators such as Trendlyne, ScanX, HDFC Sky, Business Standard, BusinessToday, Equitymaster) inside a sandboxed research session. Direct scripted/API access to the PRIMARY sources you were asked to use — screener.in, moneycontrol.com, NSE India (nseindia.com), BSE India (bseindia.com), and the companies' own Annual Report PDFs (adanipower.com, tatapower.com, torrentpower.com) — was blocked (HTTP 403) for automated fetches in this environment. All numbers not otherwise flagged therefore come from search-engine snippets of secondary coverage of those primary sources, not the primary documents themselves. UPDATE: the user subsequently uploaded the companies' actual Integrated Annual Report PDFs, and the analysis window was then NARROWED TO FY22-FY26 (the last five fiscal years) at the user's request — earlier-year data has been removed from this workbook. Within FY22-FY26, the consolidated Revenue/Total Income, PAT and Total Assets series (Sheet 2), the Ind AS 108 segment tables (Sheet 6), the AOC-1 group structure (Sheets 7-8) and the Investments detail (Sheet 9) are all PRIMARY-VERIFIED from the audited Annual Reports stored in this repo. Only the FY-end share-price rows in Sheet 2 remain to be filled (from NSE/Yahoo historical data).</t>
         </is>
       </c>
     </row>
@@ -7488,35 +7368,35 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>1. Year-end (31-Mar) share prices, FY19-FY26, all three companies — still not found for any year; pull from NSE historical data or Yahoo Finance (split-adjust Adani Power for its Sep-2025 1:5 split).</t>
+          <t>1. Year-end (31-Mar) share prices, FY22-FY26, all three companies — still not filled; pull from NSE historical data or Yahoo Finance (split-adjust Adani Power for its Sep-2025 1:5 split).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>2. Total Assets — now VERIFIED FY20-FY26 (Adani, Torrent) and FY21-FY26 (Tata) from the Annual Reports. Only FY19 (all 3) and Tata FY20 remain open (needs the FY19-20 Annual Reports).</t>
+          <t>2. Total Assets — DONE: fully VERIFIED FY22-FY26 for all three companies from the Annual Reports.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>3. Employee headcount — standalone-parent counts now VERIFIED where disclosed (Adani FY21/23/25/26; Tata FY22/23/25/26; Torrent FY21-FY26). Group-wide/consolidated headcount is still not disclosed anywhere and would be needed for a true cross-company Sales/Employee comparison.</t>
+          <t>3. Employee headcount — standalone-parent counts VERIFIED where disclosed (Adani FY23/25/26 — FY22/FY24 not disclosed in available reports; Tata FY22/23/25/26; Torrent FY22-FY26). Group-wide/consolidated headcount is not disclosed anywhere and would be needed for a true cross-company Sales/Employee comparison.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>4. Segment-wise (Ind AS 108) tables — DONE: Sheet 6 now carries verified segment revenue/results/assets for Adani Power (FY20-FY26, 2 segments) and Tata Power (FY21-FY26, 4 segments), plus the verified finding that Torrent Power reports NO segments under Ind AS 108 (single integrated business).</t>
+          <t>4. Segment-wise (Ind AS 108) tables — DONE: Sheet 6 carries verified segment revenue/results/assets for Adani Power and Tata Power (FY22-FY26), plus the verified finding that Torrent Power reports NO segments under Ind AS 108 (single integrated business).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>5. Weekly price series — DONE: 54-week adjusted-close series for all 3 stocks + Nifty 50 + Nifty Energy parsed from Yahoo HTML files in the repo; returns, volatility, and market &amp; sector betas computed in Sheet 11. Still open: year-end FY19-FY26 share prices for the Sheet 2 growth table (needs older price history).</t>
+          <t>5. Weekly price series — DONE: 54-week adjusted-close series for all 3 stocks + Nifty 50 + Nifty Energy parsed from Yahoo HTML files in the repo; returns, volatility, and market &amp; sector betas computed in Sheet 11. Still open: year-end FY22-FY26 share prices for the Sheet 2 growth table.</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7837,14 +7717,14 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>2. Growth Comparison: Sales, Assets, Profit, Market Price (FY19-FY26)</t>
+          <t>2. Growth Comparison: Sales, Assets, Profit, Market Price (FY22-FY26, last 5 years)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>₹ crore, Consolidated. FY24-FY26 columns VERIFIED from primary Annual Reports (uploaded). Yellow = still needs verification.</t>
+          <t>₹ crore, Consolidated. All columns VERIFIED from the audited Annual Reports in the repo. Yellow = still needs data.</t>
         </is>
       </c>
     </row>
@@ -7857,47 +7737,32 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>FY19</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>FY20</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="J5" s="9" t="inlineStr">
-        <is>
-          <t>CAGR</t>
+          <t>4-yr CAGR</t>
         </is>
       </c>
     </row>
@@ -7908,31 +7773,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26362</v>
+        <v>31686.47</v>
       </c>
       <c r="C7" t="n">
-        <v>27841.81</v>
+        <v>43040.52</v>
       </c>
       <c r="D7" t="n">
-        <v>28149.68</v>
+        <v>60281.48</v>
       </c>
       <c r="E7" t="n">
-        <v>31686.47</v>
+        <v>58905.83</v>
       </c>
       <c r="F7" t="n">
-        <v>43040.52</v>
-      </c>
-      <c r="G7" t="n">
-        <v>60281.48</v>
-      </c>
-      <c r="H7" t="n">
-        <v>58905.83</v>
-      </c>
-      <c r="I7" t="n">
         <v>57865.28</v>
       </c>
-      <c r="J7" s="12">
-        <f>IFERROR(IF(OR(B7="N/A",I7="N/A"),"N/A",(I7/B7)^(1/7)-1),"N/A")</f>
+      <c r="G7" s="12">
+        <f>IFERROR(IF(OR(B7="N/A",F7="N/A"),"N/A",(F7/B7)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -7943,31 +7799,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-984.4</v>
+        <v>4911.58</v>
       </c>
       <c r="C8" t="n">
-        <v>-2274.77</v>
+        <v>10726.64</v>
       </c>
       <c r="D8" t="n">
-        <v>1269.98</v>
+        <v>20828.79</v>
       </c>
       <c r="E8" t="n">
-        <v>4911.58</v>
+        <v>12749.61</v>
       </c>
       <c r="F8" t="n">
-        <v>10726.64</v>
-      </c>
-      <c r="G8" t="n">
-        <v>20828.79</v>
-      </c>
-      <c r="H8" t="n">
-        <v>12749.61</v>
-      </c>
-      <c r="I8" t="n">
         <v>12971.08</v>
       </c>
-      <c r="J8" s="12">
-        <f>IFERROR(IF(OR(B8="N/A",I8="N/A"),"N/A",(I8/B8)^(1/7)-1),"N/A")</f>
+      <c r="G8" s="12">
+        <f>IFERROR(IF(OR(B8="N/A",F8="N/A"),"N/A",(F8/B8)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -7977,34 +7824,23 @@
           <t>Adani Power — Total Assets (₹ cr)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B9" t="n">
+        <v>81981.02</v>
       </c>
       <c r="C9" t="n">
-        <v>75025</v>
+        <v>85821.27</v>
       </c>
       <c r="D9" t="n">
-        <v>78535.47</v>
+        <v>92324.77</v>
       </c>
       <c r="E9" t="n">
-        <v>81981.02</v>
+        <v>112917.57</v>
       </c>
       <c r="F9" t="n">
-        <v>85821.27</v>
-      </c>
-      <c r="G9" t="n">
-        <v>92324.77</v>
-      </c>
-      <c r="H9" t="n">
-        <v>112917.57</v>
-      </c>
-      <c r="I9" t="n">
         <v>142279.92</v>
       </c>
-      <c r="J9" s="12">
-        <f>IFERROR(IF(OR(B9="N/A",I9="N/A"),"N/A",(I9/B9)^(1/7)-1),"N/A")</f>
+      <c r="G9" s="12">
+        <f>IFERROR(IF(OR(B9="N/A",F9="N/A"),"N/A",(F9/B9)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8019,42 +7855,29 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="n">
+        <v>2805</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>84</v>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="E10" t="n">
+        <v>4210</v>
       </c>
       <c r="F10" t="n">
-        <v>2805</v>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>4210</v>
-      </c>
-      <c r="I10" t="n">
         <v>3967</v>
       </c>
-      <c r="J10" s="12">
-        <f>IFERROR(IF(OR(B10="N/A",I10="N/A"),"N/A",(I10/B10)^(1/7)-1),"N/A")</f>
+      <c r="G10" s="12">
+        <f>IFERROR(IF(OR(B10="N/A",F10="N/A"),"N/A",(F10/B10)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>FY20-FY26 figures VERIFIED from Adani Power's audited Integrated Annual Reports (consolidated). FY19 revenue/PAT are secondary-source (Business Standard, May-2019 results coverage); FY19 Total Assets not available. Employees = STANDALONE permanent employees on Company rolls: FY21's count of just 84 reflects the pre-amalgamation structure — until 1-Oct-2021 the parent was largely a holding shell, with operating staff employed by the 6 subsidiaries merged in that year, so the series has a structural break and FY21 is NOT comparable to FY23+. FY24 PAT (₹20,829cr) was inflated by one-off other income (₹9,781cr incl. prior-period revenue recognition) vs FY25's normalised ₹12,750cr.</t>
+          <t>All figures VERIFIED from Adani Power's audited Integrated Annual Reports (consolidated). Employees = STANDALONE permanent employees on Company rolls; FY22 and FY24 counts not disclosed in the reports available (the FY21-22 Annual Report is not in the repo). FY24 PAT (₹20,829cr) was inflated by one-off other income (₹9,781cr incl. prior-period revenue recognition) vs FY25's normalised ₹12,750cr.</t>
         </is>
       </c>
     </row>
@@ -8065,31 +7888,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>30743</v>
+        <v>42576</v>
       </c>
       <c r="C13" t="n">
-        <v>30350</v>
+        <v>56033</v>
       </c>
       <c r="D13" t="n">
-        <v>33239</v>
+        <v>63272.32</v>
       </c>
       <c r="E13" t="n">
-        <v>42576</v>
+        <v>66992.17</v>
       </c>
       <c r="F13" t="n">
-        <v>56033</v>
-      </c>
-      <c r="G13" t="n">
-        <v>63272.32</v>
-      </c>
-      <c r="H13" t="n">
-        <v>66992.17</v>
-      </c>
-      <c r="I13" t="n">
         <v>64171.66</v>
       </c>
-      <c r="J13" s="12">
-        <f>IFERROR(IF(OR(B13="N/A",I13="N/A"),"N/A",(I13/B13)^(1/7)-1),"N/A")</f>
+      <c r="G13" s="12">
+        <f>IFERROR(IF(OR(B13="N/A",F13="N/A"),"N/A",(F13/B13)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8099,36 +7913,23 @@
           <t>Tata Power — Net Profit / PAT (₹ cr)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B14" t="n">
+        <v>2156</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3810</v>
       </c>
       <c r="D14" t="n">
-        <v>1439</v>
+        <v>4280</v>
       </c>
       <c r="E14" t="n">
-        <v>2156</v>
+        <v>4775</v>
       </c>
       <c r="F14" t="n">
-        <v>3810</v>
-      </c>
-      <c r="G14" t="n">
-        <v>4280</v>
-      </c>
-      <c r="H14" t="n">
-        <v>4775</v>
-      </c>
-      <c r="I14" t="n">
         <v>5118</v>
       </c>
-      <c r="J14" s="12">
-        <f>IFERROR(IF(OR(B14="N/A",I14="N/A"),"N/A",(I14/B14)^(1/7)-1),"N/A")</f>
+      <c r="G14" s="12">
+        <f>IFERROR(IF(OR(B14="N/A",F14="N/A"),"N/A",(F14/B14)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8138,36 +7939,23 @@
           <t>Tata Power — Total Assets (₹ cr)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B15" t="n">
+        <v>112884.59</v>
+      </c>
+      <c r="C15" t="n">
+        <v>128349.04</v>
       </c>
       <c r="D15" t="n">
-        <v>98838.86</v>
+        <v>139553.49</v>
       </c>
       <c r="E15" t="n">
-        <v>112884.59</v>
+        <v>156711.29</v>
       </c>
       <c r="F15" t="n">
-        <v>128349.04</v>
-      </c>
-      <c r="G15" t="n">
-        <v>139553.49</v>
-      </c>
-      <c r="H15" t="n">
-        <v>156711.29</v>
-      </c>
-      <c r="I15" t="n">
         <v>175171.78</v>
       </c>
-      <c r="J15" s="12">
-        <f>IFERROR(IF(OR(B15="N/A",I15="N/A"),"N/A",(I15/B15)^(1/7)-1),"N/A")</f>
+      <c r="G15" s="12">
+        <f>IFERROR(IF(OR(B15="N/A",F15="N/A"),"N/A",(F15/B15)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8177,47 +7965,32 @@
           <t>Tata Power — Employees (#)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="n">
+        <v>2815</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3071</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E16" t="n">
-        <v>2815</v>
+        <v>3130</v>
       </c>
       <c r="F16" t="n">
-        <v>3071</v>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>3130</v>
-      </c>
-      <c r="I16" t="n">
         <v>3295</v>
       </c>
-      <c r="J16" s="12">
-        <f>IFERROR(IF(OR(B16="N/A",I16="N/A"),"N/A",(I16/B16)^(1/7)-1),"N/A")</f>
+      <c r="G16" s="12">
+        <f>IFERROR(IF(OR(B16="N/A",F16="N/A"),"N/A",(F16/B16)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>FY21-FY26 figures VERIFIED from Tata Power's Integrated Annual Reports (consolidated, reported basis): PAT FY21 ₹1,439cr / FY22 ₹2,156cr / FY23 ₹3,810cr replace earlier secondary-source variants (1,424/2,298/3,878, which were pre-exceptional or pre-minority-interest bases). Revenue FY21-23 (33,239/42,576/56,033) is the company's own highlights-basis series incl. regulatory income, now confirmed in the FY22/FY23 Annual Reports; as-reported P&amp;L 'Revenue from Operations' is slightly lower (32,703/42,816/55,109). FY19/FY20 figures remain secondary-source. Employees = STANDALONE parent only (~2,800-3,300) — most of the group workforce sits in subsidiaries (TPREL, discoms), so do not compare with consolidated revenue.</t>
+          <t>All figures VERIFIED from Tata Power's Integrated Annual Reports (consolidated, reported basis). Revenue FY22-23 (42,576/56,033) is the company's own highlights-basis series incl. regulatory income; as-reported P&amp;L 'Revenue from Operations' is slightly lower (42,816/55,109). Employees = STANDALONE parent only (~2,800-3,300) — most of the group workforce sits in subsidiaries (TPREL, discoms), so do not compare with consolidated revenue.</t>
         </is>
       </c>
     </row>
@@ -8227,34 +8000,23 @@
           <t>Torrent Power — Revenue / Total Income (₹ cr)</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B19" t="n">
+        <v>14492.65</v>
       </c>
       <c r="C19" t="n">
-        <v>13818.22</v>
+        <v>26075.97</v>
       </c>
       <c r="D19" t="n">
-        <v>12314.47</v>
+        <v>27527.53</v>
       </c>
       <c r="E19" t="n">
-        <v>14492.65</v>
+        <v>29652.47</v>
       </c>
       <c r="F19" t="n">
-        <v>26075.97</v>
-      </c>
-      <c r="G19" t="n">
-        <v>27527.53</v>
-      </c>
-      <c r="H19" t="n">
-        <v>29652.47</v>
-      </c>
-      <c r="I19" t="n">
         <v>29288.92</v>
       </c>
-      <c r="J19" s="12">
-        <f>IFERROR(IF(OR(B19="N/A",I19="N/A"),"N/A",(I19/B19)^(1/7)-1),"N/A")</f>
+      <c r="G19" s="12">
+        <f>IFERROR(IF(OR(B19="N/A",F19="N/A"),"N/A",(F19/B19)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8264,34 +8026,23 @@
           <t>Torrent Power — Net Profit / PAT (₹ cr)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B20" t="n">
+        <v>458.7</v>
       </c>
       <c r="C20" t="n">
-        <v>1178.88</v>
+        <v>2164.67</v>
       </c>
       <c r="D20" t="n">
-        <v>1295.87</v>
+        <v>1896</v>
       </c>
       <c r="E20" t="n">
-        <v>458.7</v>
+        <v>3058.61</v>
       </c>
       <c r="F20" t="n">
-        <v>2164.67</v>
-      </c>
-      <c r="G20" t="n">
-        <v>1896</v>
-      </c>
-      <c r="H20" t="n">
-        <v>3058.61</v>
-      </c>
-      <c r="I20" t="n">
         <v>2469.36</v>
       </c>
-      <c r="J20" s="12">
-        <f>IFERROR(IF(OR(B20="N/A",I20="N/A"),"N/A",(I20/B20)^(1/7)-1),"N/A")</f>
+      <c r="G20" s="12">
+        <f>IFERROR(IF(OR(B20="N/A",F20="N/A"),"N/A",(F20/B20)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8301,34 +8052,23 @@
           <t>Torrent Power — Total Assets (₹ cr)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B21" t="n">
+        <v>25022.7</v>
       </c>
       <c r="C21" t="n">
-        <v>23623.04</v>
+        <v>29910.18</v>
       </c>
       <c r="D21" t="n">
-        <v>23538.72</v>
+        <v>33392.48</v>
       </c>
       <c r="E21" t="n">
-        <v>25022.7</v>
+        <v>36573.38</v>
       </c>
       <c r="F21" t="n">
-        <v>29910.18</v>
-      </c>
-      <c r="G21" t="n">
-        <v>33392.48</v>
-      </c>
-      <c r="H21" t="n">
-        <v>36573.38</v>
-      </c>
-      <c r="I21" t="n">
         <v>45193.28</v>
       </c>
-      <c r="J21" s="12">
-        <f>IFERROR(IF(OR(B21="N/A",I21="N/A"),"N/A",(I21/B21)^(1/7)-1),"N/A")</f>
+      <c r="G21" s="12">
+        <f>IFERROR(IF(OR(B21="N/A",F21="N/A"),"N/A",(F21/B21)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -8338,43 +8078,30 @@
           <t>Torrent Power — Employees (#)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B22" t="n">
+        <v>7603</v>
+      </c>
+      <c r="C22" t="n">
+        <v>6992</v>
       </c>
       <c r="D22" t="n">
-        <v>7429</v>
+        <v>6987</v>
       </c>
       <c r="E22" t="n">
-        <v>7603</v>
+        <v>7213</v>
       </c>
       <c r="F22" t="n">
-        <v>6992</v>
-      </c>
-      <c r="G22" t="n">
-        <v>6987</v>
-      </c>
-      <c r="H22" t="n">
-        <v>7213</v>
-      </c>
-      <c r="I22" t="n">
         <v>6687</v>
       </c>
-      <c r="J22" s="12">
-        <f>IFERROR(IF(OR(B22="N/A",I22="N/A"),"N/A",(I22/B22)^(1/7)-1),"N/A")</f>
+      <c r="G22" s="12">
+        <f>IFERROR(IF(OR(B22="N/A",F22="N/A"),"N/A",(F22/B22)^(1/4)-1),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>FY20-FY26 figures VERIFIED from Torrent Power's Integrated Annual Reports (consolidated). Only FY19 remains unverified (no FY19-20 report uploaded). FY22 PAT (₹458.70cr) was depressed by a ~₹1,300cr DGEN plant impairment. Employees = standalone permanent employees on Company rolls (Rule 5(1) disclosure) — Torrent runs most operations in the parent entity, so this series is closer to a true group headcount than Adani/Tata's standalone counts.</t>
+          <t>All figures VERIFIED from Torrent Power's Integrated Annual Reports (consolidated). FY22 PAT (₹458.70cr) was depressed by a ~₹1,300cr DGEN plant impairment — treat FY22-base growth rates with care. Employees = standalone permanent employees on Company rolls (Rule 5(1) disclosure) — Torrent runs most operations in the parent entity, so this series is closer to a true group headcount than Adani/Tata's standalone counts.</t>
         </is>
       </c>
     </row>
@@ -8416,21 +8143,6 @@
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8463,21 +8175,6 @@
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8510,21 +8207,6 @@
           <t>TO FILL</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>TO FILL</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
@@ -8536,7 +8218,7 @@
     <row r="31" ht="100" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>SALES GROWTH: Adani Power's revenue rose from ₹27,842cr (FY20) to ₹57,865cr (FY26), ~13% CAGR, with the big jumps in FY23-FY24 driven by IBC acquisitions (Mahan, Korba) plus tariff/prior-period recoveries; FY25-FY26 revenue plateaued. Tata Power roughly doubled revenue FY20→FY26 (₹30,350cr→₹64,172cr), the FY22-23 surge reflecting the four Odisha discoms and high Mundra fuel pass-throughs. Torrent Power's revenue more than doubled (₹13,818cr→₹29,289cr), with the single biggest step in FY23 (+80%) from the DNH&amp;DD discom takeover and merchant gas sales. PROFIT GROWTH: Adani Power's swing is the most dramatic — from a ₹2,275cr loss (FY20) to ₹12,971cr PAT (FY26); FY24's ₹20,829cr spike was one-off-boosted and FY25/FY26 is the cleaner run-rate. Tata Power compounded PAT steadily every single year (₹1,439cr FY21 → ₹5,118cr FY26, ~29% CAGR) — the most consistent grower. Torrent is profitable but lumpy (FY22 impairment, FY25 peak, FY26 dip). ASSETS GROWTH: Adani Power's asset base compounded ~11% (₹75,025cr FY20 → ₹1,42,280cr FY26), accelerating sharply after FY24 as acquisitions/new capacity landed. Tata Power grew assets ~12% CAGR (₹98,839cr FY21 → ₹1,75,172cr FY26) — the largest absolute base. Torrent was static FY20-FY22 (~₹23-25,000cr) then accelerated to ₹45,193cr by FY26 (Nabha + capex cycle). MARKET PRICE: year-end share-price rows still need NSE/Yahoo data (yellow) to complete the fourth growth lens.</t>
+          <t>SALES GROWTH (FY22→FY26): Adani Power grew revenue ~83% (₹31,686cr → ₹57,865cr, ~16% CAGR), driven by IBC acquisitions (Mahan, Korba) and tariff/prior-period recoveries in FY23-FY24, before plateauing in FY25-FY26. Torrent Power doubled revenue (₹14,493cr → ₹29,289cr, ~19% CAGR) with the single biggest step in FY23 (+80%) from the DNH&amp;DD discom takeover and merchant gas sales. Tata Power grew ~51% (₹42,576cr → ₹64,172cr, ~11% CAGR). PROFIT GROWTH: Adani Power PAT rose from ₹4,912cr to ₹12,971cr (~27% CAGR); FY24's ₹20,829cr spike was one-off-boosted and FY25/FY26 is the cleaner run-rate. Tata Power compounded PAT steadily every single year (₹2,156cr → ₹5,118cr, ~24% CAGR) — the most consistent grower. Torrent is profitable but lumpy: FY22 was impairment-depressed (₹459cr), rebounding to ₹2,165-3,059cr, easing to ₹2,469cr in FY26. ASSETS GROWTH: Adani Power's asset base grew ~74% (₹81,981cr → ₹1,42,280cr), accelerating sharply after FY24 as acquisitions and new capacity landed. Tata Power grew ~55% to ₹1,75,172cr — the largest absolute base. Torrent grew ~81% (₹25,023cr → ₹45,193cr; Nabha Power + capex cycle) — the fastest in relative terms. MARKET PRICE: year-end share-price rows still need NSE/Yahoo historical data (yellow) to complete the fourth lens.</t>
         </is>
       </c>
     </row>
@@ -8546,12 +8228,12 @@
     <row r="35"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A31:J35"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A31:G35"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8565,7 +8247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8593,397 +8275,284 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FY19</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26362</v>
+        <v>31686.47</v>
       </c>
       <c r="C2" t="n">
-        <v>30743</v>
+        <v>42576</v>
+      </c>
+      <c r="D2" t="n">
+        <v>14492.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FY20</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>27841.81</v>
+        <v>43040.52</v>
       </c>
       <c r="C3" t="n">
-        <v>30350</v>
+        <v>56033</v>
       </c>
       <c r="D3" t="n">
-        <v>13818.22</v>
+        <v>26075.97</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>28149.68</v>
+        <v>60281.48</v>
       </c>
       <c r="C4" t="n">
-        <v>33239</v>
+        <v>63272.32</v>
       </c>
       <c r="D4" t="n">
-        <v>12314.47</v>
+        <v>27527.53</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31686.47</v>
+        <v>58905.83</v>
       </c>
       <c r="C5" t="n">
-        <v>42576</v>
+        <v>66992.17</v>
       </c>
       <c r="D5" t="n">
-        <v>14492.65</v>
+        <v>29652.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>43040.52</v>
+        <v>57865.28</v>
       </c>
       <c r="C6" t="n">
-        <v>56033</v>
+        <v>64171.66</v>
       </c>
       <c r="D6" t="n">
-        <v>26075.97</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>60281.48</v>
-      </c>
-      <c r="C7" t="n">
-        <v>63272.32</v>
-      </c>
-      <c r="D7" t="n">
-        <v>27527.53</v>
+        <v>29288.92</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>58905.83</v>
-      </c>
-      <c r="C8" t="n">
-        <v>66992.17</v>
-      </c>
-      <c r="D8" t="n">
-        <v>29652.47</v>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Adani Power PAT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tata Power PAT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Torrent Power PAT</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>57865.28</v>
+        <v>4911.58</v>
       </c>
       <c r="C9" t="n">
-        <v>64171.66</v>
+        <v>2156</v>
       </c>
       <c r="D9" t="n">
-        <v>29288.92</v>
+        <v>458.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FY23</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10726.64</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3810</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2164.67</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Adani Power PAT</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Tata Power PAT</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Torrent Power PAT</t>
-        </is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20828.79</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4280</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1896</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FY19</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-984.4</v>
+        <v>12749.61</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4775</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3058.61</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FY20</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-2274.77</v>
+        <v>12971.08</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5118</v>
       </c>
       <c r="D13" t="n">
-        <v>1178.88</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>FY21</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1269.98</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1439</v>
-      </c>
-      <c r="D14" t="n">
-        <v>1295.87</v>
+        <v>2469.36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>4911.58</v>
-      </c>
-      <c r="C15" t="n">
-        <v>2156</v>
-      </c>
-      <c r="D15" t="n">
-        <v>458.7</v>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Adani Power Assets</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tata Power Assets</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Torrent Power Assets</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>10726.64</v>
+        <v>81981.02</v>
       </c>
       <c r="C16" t="n">
-        <v>3810</v>
+        <v>112884.59</v>
       </c>
       <c r="D16" t="n">
-        <v>2164.67</v>
+        <v>25022.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>20828.79</v>
+        <v>85821.27</v>
       </c>
       <c r="C17" t="n">
-        <v>4280</v>
+        <v>128349.04</v>
       </c>
       <c r="D17" t="n">
-        <v>1896</v>
+        <v>29910.18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12749.61</v>
+        <v>92324.77</v>
       </c>
       <c r="C18" t="n">
-        <v>4775</v>
+        <v>139553.49</v>
       </c>
       <c r="D18" t="n">
-        <v>3058.61</v>
+        <v>33392.48</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>112917.57</v>
+      </c>
+      <c r="C19" t="n">
+        <v>156711.29</v>
+      </c>
+      <c r="D19" t="n">
+        <v>36573.38</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>FY26</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>12971.08</v>
-      </c>
-      <c r="C19" t="n">
-        <v>5118</v>
-      </c>
-      <c r="D19" t="n">
-        <v>2469.36</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Adani Power Assets</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Tata Power Assets</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Torrent Power Assets</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>FY20</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>75025</v>
-      </c>
-      <c r="D22" t="n">
-        <v>23623.04</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FY21</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>78535.47</v>
-      </c>
-      <c r="C23" t="n">
-        <v>98838.86</v>
-      </c>
-      <c r="D23" t="n">
-        <v>23538.72</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>81981.02</v>
-      </c>
-      <c r="C24" t="n">
-        <v>112884.59</v>
-      </c>
-      <c r="D24" t="n">
-        <v>25022.7</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>85821.27</v>
-      </c>
-      <c r="C25" t="n">
-        <v>128349.04</v>
-      </c>
-      <c r="D25" t="n">
-        <v>29910.18</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>92324.77</v>
-      </c>
-      <c r="C26" t="n">
-        <v>139553.49</v>
-      </c>
-      <c r="D26" t="n">
-        <v>33392.48</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>112917.57</v>
-      </c>
-      <c r="C27" t="n">
-        <v>156711.29</v>
-      </c>
-      <c r="D27" t="n">
-        <v>36573.38</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
+      <c r="B20" t="n">
         <v>142279.92</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C20" t="n">
         <v>175171.78</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D20" t="n">
         <v>45193.28</v>
       </c>
     </row>
@@ -8998,24 +8567,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>3. Sales per Rupee of Asset Deployed &amp; Sales per Employee</t>
+          <t>3. Sales per Rupee of Asset Deployed &amp; Sales per Employee (FY22-FY26)</t>
         </is>
       </c>
     </row>
@@ -9035,40 +8601,25 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>FY19</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>FY20</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
@@ -9100,18 +8651,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F7),ISTEXT('2_Growth_Comparison'!F9)),"N/A",'2_Growth_Comparison'!F7/'2_Growth_Comparison'!F9),"N/A")</f>
         <v/>
       </c>
-      <c r="G7" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G7),ISTEXT('2_Growth_Comparison'!G9)),"N/A",'2_Growth_Comparison'!G7/'2_Growth_Comparison'!G9),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H7" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H7),ISTEXT('2_Growth_Comparison'!H9)),"N/A",'2_Growth_Comparison'!H7/'2_Growth_Comparison'!H9),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I7" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I7),ISTEXT('2_Growth_Comparison'!I9)),"N/A",'2_Growth_Comparison'!I7/'2_Growth_Comparison'!I9),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9139,18 +8678,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F7),ISTEXT('2_Growth_Comparison'!F10)),"N/A",'2_Growth_Comparison'!F7*100/'2_Growth_Comparison'!F10),"N/A")</f>
         <v/>
       </c>
-      <c r="G8" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G7),ISTEXT('2_Growth_Comparison'!G10)),"N/A",'2_Growth_Comparison'!G7*100/'2_Growth_Comparison'!G10),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H8" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H7),ISTEXT('2_Growth_Comparison'!H10)),"N/A",'2_Growth_Comparison'!H7*100/'2_Growth_Comparison'!H10),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I8" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I7),ISTEXT('2_Growth_Comparison'!I10)),"N/A",'2_Growth_Comparison'!I7*100/'2_Growth_Comparison'!I10),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -9178,18 +8705,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F13),ISTEXT('2_Growth_Comparison'!F15)),"N/A",'2_Growth_Comparison'!F13/'2_Growth_Comparison'!F15),"N/A")</f>
         <v/>
       </c>
-      <c r="G10" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G13),ISTEXT('2_Growth_Comparison'!G15)),"N/A",'2_Growth_Comparison'!G13/'2_Growth_Comparison'!G15),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H10" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H13),ISTEXT('2_Growth_Comparison'!H15)),"N/A",'2_Growth_Comparison'!H13/'2_Growth_Comparison'!H15),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I10" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I13),ISTEXT('2_Growth_Comparison'!I15)),"N/A",'2_Growth_Comparison'!I13/'2_Growth_Comparison'!I15),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -9217,18 +8732,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F13),ISTEXT('2_Growth_Comparison'!F16)),"N/A",'2_Growth_Comparison'!F13*100/'2_Growth_Comparison'!F16),"N/A")</f>
         <v/>
       </c>
-      <c r="G11" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G13),ISTEXT('2_Growth_Comparison'!G16)),"N/A",'2_Growth_Comparison'!G13*100/'2_Growth_Comparison'!G16),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H11" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H13),ISTEXT('2_Growth_Comparison'!H16)),"N/A",'2_Growth_Comparison'!H13*100/'2_Growth_Comparison'!H16),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I11" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I13),ISTEXT('2_Growth_Comparison'!I16)),"N/A",'2_Growth_Comparison'!I13*100/'2_Growth_Comparison'!I16),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -9256,18 +8759,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F19),ISTEXT('2_Growth_Comparison'!F21)),"N/A",'2_Growth_Comparison'!F19/'2_Growth_Comparison'!F21),"N/A")</f>
         <v/>
       </c>
-      <c r="G13" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G19),ISTEXT('2_Growth_Comparison'!G21)),"N/A",'2_Growth_Comparison'!G19/'2_Growth_Comparison'!G21),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H13" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H19),ISTEXT('2_Growth_Comparison'!H21)),"N/A",'2_Growth_Comparison'!H19/'2_Growth_Comparison'!H21),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I13" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I19),ISTEXT('2_Growth_Comparison'!I21)),"N/A",'2_Growth_Comparison'!I19/'2_Growth_Comparison'!I21),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -9295,18 +8786,6 @@
         <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!F19),ISTEXT('2_Growth_Comparison'!F22)),"N/A",'2_Growth_Comparison'!F19*100/'2_Growth_Comparison'!F22),"N/A")</f>
         <v/>
       </c>
-      <c r="G14" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!G19),ISTEXT('2_Growth_Comparison'!G22)),"N/A",'2_Growth_Comparison'!G19*100/'2_Growth_Comparison'!G22),"N/A")</f>
-        <v/>
-      </c>
-      <c r="H14" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!H19),ISTEXT('2_Growth_Comparison'!H22)),"N/A",'2_Growth_Comparison'!H19*100/'2_Growth_Comparison'!H22),"N/A")</f>
-        <v/>
-      </c>
-      <c r="I14" s="17">
-        <f>IFERROR(IF(OR(ISTEXT('2_Growth_Comparison'!I19),ISTEXT('2_Growth_Comparison'!I22)),"N/A",'2_Growth_Comparison'!I19*100/'2_Growth_Comparison'!I22),"N/A")</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -9318,7 +8797,7 @@
     <row r="17" ht="130" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>SALES PER RUPEE OF ASSET (now computable FY20/FY21-FY26 from verified Annual Report data): Adani Power improved from ~0.37x (FY20, low utilisation/losses era) to a peak of ~0.65x (FY24), then fell back to ~0.41x (FY26) as its asset base ballooned ahead of revenue from new acquisitions still ramping up. Tata Power is stable in a ~0.34-0.45x band — typical of a regulated, asset-heavy integrated utility. Torrent Power is consistently the MOST asset-efficient of the three (~0.52-0.87x, peaking FY23 when DNH&amp;DD volumes hit a still-small asset base) — its regulated distribution business generates more revenue per rupee of assets than pure thermal generation does. SALES PER EMPLOYEE: comparable across time within Torrent (parent employs most staff: ~₹18-44 cr/employee trend) but NOT comparable across companies — Adani and Tata employee counts are standalone-parent only, while their revenue is consolidated (Tata's discoms/TPREL staff and Adani's pre-FY22 plant staff sit in subsidiaries). Adani's FY21 count of 84 (pre-amalgamation shell) makes that year's ratio meaningless and it is excluded from comment. Use the Torrent series as the benchmark and treat Adani/Tata Sales-per-Employee as indicative only, noting the basis in any write-up.</t>
+          <t>SALES PER RUPEE OF ASSET (all five years computed from verified Annual Report data): Adani Power improved from ~0.39x (FY22) to a peak of ~0.65x (FY24), then fell back to ~0.41x (FY26) as its asset base ballooned ahead of revenue from new acquisitions still ramping up. Tata Power is stable in a ~0.37-0.45x band — typical of a regulated, asset-heavy integrated utility. Torrent Power is consistently the MOST asset-efficient of the three (~0.58-0.87x, peaking FY23 when DNH&amp;DD volumes hit a still-small asset base) — its regulated distribution business generates more revenue per rupee of assets than pure thermal generation does. SALES PER EMPLOYEE: comparable across time within Torrent (parent employs most staff) but NOT comparable across companies — Adani and Tata employee counts are standalone-parent only, while their revenue is consolidated (Tata's discoms/TPREL staff sit in subsidiaries). Use the Torrent series as the benchmark and treat Adani/Tata Sales-per-Employee as indicative only, noting the basis in any write-up.</t>
         </is>
       </c>
     </row>
@@ -9331,9 +8810,9 @@
     <row r="24"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A17:I24"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10370,7 +9849,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>₹ crore, consolidated. Extracted directly from the 'Segment Reporting' notes of each company's audited Annual Reports (FY21-FY26 reports uploaded by user).</t>
+          <t>₹ crore, consolidated, FY22-FY26. Extracted directly from the 'Segment Reporting' notes of each company's audited Annual Reports.</t>
         </is>
       </c>
     </row>
@@ -10390,35 +9869,25 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>FY20</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
@@ -10431,24 +9900,18 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>26005.92</v>
+        <v>27221.78</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>25870.6</v>
+        <v>37895.85</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>27221.78</v>
+        <v>50014.16</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>37895.85</v>
+        <v>56107.06</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>50014.16</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>56107.06</v>
-      </c>
-      <c r="H7" s="19" t="n">
         <v>54240.52</v>
       </c>
     </row>
@@ -10459,24 +9922,18 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>461.8</v>
+        <v>489.4</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>350.88</v>
+        <v>877.45</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>489.4</v>
+        <v>337.09</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>877.45</v>
+        <v>96.03</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>337.09</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>96.03</v>
-      </c>
-      <c r="H8" s="19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10486,29 +9943,19 @@
           <t>Segment Results — Power Generation</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B9" s="19" t="n">
+        <v>6571.37</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>6957.13</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>6571.37</v>
+        <v>20557.22</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>6957.13</v>
+        <v>16540.39</v>
       </c>
       <c r="F9" s="19" t="n">
-        <v>20557.22</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>16540.39</v>
-      </c>
-      <c r="H9" s="19" t="n">
         <v>15757.55</v>
       </c>
     </row>
@@ -10518,29 +9965,19 @@
           <t>Segment Results — Trading/Investment/Other</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="B10" s="19" t="n">
+        <v>5.76</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>717.5700000000001</v>
       </c>
       <c r="D10" s="19" t="n">
-        <v>5.76</v>
+        <v>234.29</v>
       </c>
       <c r="E10" s="19" t="n">
-        <v>717.5700000000001</v>
+        <v>-1.81</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>234.29</v>
-      </c>
-      <c r="G10" s="19" t="n">
-        <v>-1.81</v>
-      </c>
-      <c r="H10" s="19" t="n">
         <v>13.68</v>
       </c>
     </row>
@@ -10551,24 +9988,18 @@
         </is>
       </c>
       <c r="B11" s="19" t="n">
-        <v>74847.53999999999</v>
+        <v>81888.09</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>77747</v>
+        <v>84364.22</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>81888.09</v>
+        <v>91378.85000000001</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>84364.22</v>
+        <v>111162.48</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>91378.85000000001</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>111162.48</v>
-      </c>
-      <c r="H11" s="19" t="n">
         <v>139777.31</v>
       </c>
     </row>
@@ -10579,31 +10010,25 @@
         </is>
       </c>
       <c r="B12" s="19" t="n">
-        <v>177.46</v>
+        <v>42.02</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>788.47</v>
+        <v>1134.26</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>42.02</v>
+        <v>203.86</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>1134.26</v>
+        <v>1328.18</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>203.86</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>1328.18</v>
-      </c>
-      <c r="H12" s="19" t="n">
         <v>1354.52</v>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>FY20/21 segment results shown as N/A because the FY21 report used a different basis ('profit before interest…', not comparable); FY22-23 results are as restated in the FY23 report after a CODM methodology change. FY26 Trading revenue was nil; segment results shown are pre-tax basis per each year's note.</t>
+          <t>FY22-23 results are as restated in the FY23 report after a CODM methodology change. FY26 Trading revenue was nil; segment results shown are pre-tax basis per each year's note.</t>
         </is>
       </c>
     </row>
@@ -10622,30 +10047,25 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>FY26</t>
         </is>
@@ -10658,21 +10078,18 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>13432.77</v>
+        <v>11211.03</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>11211.03</v>
+        <v>18211.35</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>18211.35</v>
+        <v>19613.61</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>19613.61</v>
+        <v>19739.07</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>19739.07</v>
-      </c>
-      <c r="G17" s="19" t="n">
         <v>11635.93</v>
       </c>
     </row>
@@ -10683,21 +10100,18 @@
         </is>
       </c>
       <c r="B18" s="19" t="n">
-        <v>5887.65</v>
+        <v>7748.9</v>
       </c>
       <c r="C18" s="19" t="n">
-        <v>7748.9</v>
+        <v>8196.91</v>
       </c>
       <c r="D18" s="19" t="n">
-        <v>8196.91</v>
+        <v>10175.29</v>
       </c>
       <c r="E18" s="19" t="n">
-        <v>10175.29</v>
+        <v>9876.360000000001</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>9876.360000000001</v>
-      </c>
-      <c r="G18" s="19" t="n">
         <v>15027.82</v>
       </c>
     </row>
@@ -10708,21 +10122,18 @@
         </is>
       </c>
       <c r="B19" s="19" t="n">
-        <v>16829.85</v>
+        <v>27493.17</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>27493.17</v>
+        <v>34529.36</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>34529.36</v>
+        <v>36205.82</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>36205.82</v>
+        <v>39120.52</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>39120.52</v>
-      </c>
-      <c r="G19" s="19" t="n">
         <v>41338.59</v>
       </c>
     </row>
@@ -10733,21 +10144,18 @@
         </is>
       </c>
       <c r="B20" s="19" t="n">
-        <v>262.16</v>
+        <v>317.8</v>
       </c>
       <c r="C20" s="19" t="n">
-        <v>317.8</v>
+        <v>413.56</v>
       </c>
       <c r="D20" s="19" t="n">
-        <v>413.56</v>
+        <v>430.62</v>
       </c>
       <c r="E20" s="19" t="n">
-        <v>430.62</v>
+        <v>431.04</v>
       </c>
       <c r="F20" s="19" t="n">
-        <v>431.04</v>
-      </c>
-      <c r="G20" s="19" t="n">
         <v>431.79</v>
       </c>
     </row>
@@ -10758,21 +10166,18 @@
         </is>
       </c>
       <c r="B21" s="19" t="n">
-        <v>2709.81</v>
+        <v>2632.75</v>
       </c>
       <c r="C21" s="19" t="n">
-        <v>2632.75</v>
+        <v>5092.16</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>5092.16</v>
+        <v>2569.61</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>2569.61</v>
+        <v>2878.91</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>2878.91</v>
-      </c>
-      <c r="G21" s="19" t="n">
         <v>1137.94</v>
       </c>
     </row>
@@ -10783,21 +10188,18 @@
         </is>
       </c>
       <c r="B22" s="19" t="n">
-        <v>1494.25</v>
+        <v>1923.57</v>
       </c>
       <c r="C22" s="19" t="n">
-        <v>1923.57</v>
+        <v>1932.01</v>
       </c>
       <c r="D22" s="19" t="n">
-        <v>1932.01</v>
+        <v>2147.1</v>
       </c>
       <c r="E22" s="19" t="n">
-        <v>2147.1</v>
+        <v>2880.68</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>2880.68</v>
-      </c>
-      <c r="G22" s="19" t="n">
         <v>4340.93</v>
       </c>
     </row>
@@ -10808,21 +10210,18 @@
         </is>
       </c>
       <c r="B23" s="19" t="n">
-        <v>1677.02</v>
+        <v>2138.49</v>
       </c>
       <c r="C23" s="19" t="n">
-        <v>2138.49</v>
+        <v>2197.68</v>
       </c>
       <c r="D23" s="19" t="n">
-        <v>2197.68</v>
+        <v>2418.22</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>2418.22</v>
+        <v>3128.27</v>
       </c>
       <c r="F23" s="19" t="n">
-        <v>3128.27</v>
-      </c>
-      <c r="G23" s="19" t="n">
         <v>4307.95</v>
       </c>
     </row>
@@ -10833,21 +10232,18 @@
         </is>
       </c>
       <c r="B24" s="19" t="n">
-        <v>83.16</v>
+        <v>-286.03</v>
       </c>
       <c r="C24" s="19" t="n">
-        <v>-286.03</v>
+        <v>-308.17</v>
       </c>
       <c r="D24" s="19" t="n">
-        <v>-308.17</v>
+        <v>105.38</v>
       </c>
       <c r="E24" s="19" t="n">
-        <v>105.38</v>
+        <v>112.8</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>112.8</v>
-      </c>
-      <c r="G24" s="19" t="n">
         <v>104.72</v>
       </c>
     </row>
@@ -10858,21 +10254,18 @@
         </is>
       </c>
       <c r="B25" s="19" t="n">
-        <v>37717.32</v>
+        <v>38201.93</v>
       </c>
       <c r="C25" s="19" t="n">
-        <v>38201.93</v>
+        <v>41201.04</v>
       </c>
       <c r="D25" s="19" t="n">
-        <v>41201.04</v>
+        <v>39315.88</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>39315.88</v>
+        <v>39708.11</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>39708.11</v>
-      </c>
-      <c r="G25" s="19" t="n">
         <v>41697.31</v>
       </c>
     </row>
@@ -10883,21 +10276,18 @@
         </is>
       </c>
       <c r="B26" s="19" t="n">
-        <v>22702.98</v>
+        <v>27589.28</v>
       </c>
       <c r="C26" s="19" t="n">
-        <v>27589.28</v>
+        <v>29744.49</v>
       </c>
       <c r="D26" s="19" t="n">
-        <v>29744.49</v>
+        <v>40459.25</v>
       </c>
       <c r="E26" s="19" t="n">
-        <v>40459.25</v>
+        <v>51355.61</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>51355.61</v>
-      </c>
-      <c r="G26" s="19" t="n">
         <v>56921.28</v>
       </c>
     </row>
@@ -10908,21 +10298,18 @@
         </is>
       </c>
       <c r="B27" s="19" t="n">
-        <v>25542.61</v>
+        <v>32411.34</v>
       </c>
       <c r="C27" s="19" t="n">
-        <v>32411.34</v>
+        <v>37477.26</v>
       </c>
       <c r="D27" s="19" t="n">
-        <v>37477.26</v>
+        <v>42059.9</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>42059.9</v>
+        <v>45707.75</v>
       </c>
       <c r="F27" s="19" t="n">
-        <v>45707.75</v>
-      </c>
-      <c r="G27" s="19" t="n">
         <v>53428.87</v>
       </c>
     </row>
@@ -10933,21 +10320,18 @@
         </is>
       </c>
       <c r="B28" s="19" t="n">
-        <v>12875.95</v>
+        <v>14682.04</v>
       </c>
       <c r="C28" s="19" t="n">
-        <v>14682.04</v>
+        <v>19926.25</v>
       </c>
       <c r="D28" s="19" t="n">
-        <v>19926.25</v>
+        <v>17718.46</v>
       </c>
       <c r="E28" s="19" t="n">
-        <v>17718.46</v>
+        <v>19939.82</v>
       </c>
       <c r="F28" s="19" t="n">
-        <v>19939.82</v>
-      </c>
-      <c r="G28" s="19" t="n">
         <v>23124.32</v>
       </c>
     </row>
@@ -10986,7 +10370,7 @@
     <row r="39" ht="150" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>GENERATION is the only segment where all three effectively compete, and the verified numbers show a stark contrast: Adani Power's generation segment grew revenue ~2.1x (₹26,006cr FY20 → ₹54,241cr FY26) with segment results of ₹15,758-20,557cr in FY24-26 — vastly more profitable than Tata Power's generation segment (results of only ₹1,138-2,879cr on ₹11,636-19,739cr revenue in the same years, dragged by the Mundra plant's fuel economics and eventual shutdown). Adani is unambiguously the generation winner. RENEWABLES: only Tata Power reports it separately, and it is now their growth engine — revenue up 2.6x (₹5,888cr FY21 → ₹15,028cr FY26), results up 2.9x (₹1,494cr → ₹4,341cr), and segment assets up 2.5x to ₹56,921cr, overtaking every other Tata segment. Adani Power has no renewables segment (that sits in sister company Adani Green). TRANSMISSION &amp; DISTRIBUTION: Tata Power's largest and steadiest segment — revenue grew ₹16,830cr → ₹41,339cr (FY21→FY26, boosted by the Odisha discoms) with consistently positive, regulated-return results (₹1,677cr → ₹4,308cr). Torrent's distribution business is economically similar (regulated, stable) but not separately reported. INDUSTRY CONTEXT: India's power demand grew ~7-8%/yr (CEA) over this period — Adani's generation growth (~13% CAGR) and Tata's renewables growth (~21% CAGR) both outpaced the sector, largely through acquisitions and capacity build-out respectively, while Tata's generation segment underperformed the sector.</t>
+          <t>GENERATION is the only segment where all three effectively compete, and the verified numbers show a stark contrast: Adani Power's generation segment grew revenue ~2.0x (₹27,222cr FY22 → ₹54,241cr FY26) with segment results of ₹15,758-20,557cr in FY24-26 — vastly more profitable than Tata Power's generation segment (results of only ₹1,138-2,879cr on ₹11,636-19,739cr revenue in the same years, dragged by the Mundra plant's fuel economics and eventual shutdown). Adani is unambiguously the generation winner. RENEWABLES: only Tata Power reports it separately, and it is now their growth engine — revenue up ~1.9x (₹7,749cr FY22 → ₹15,028cr FY26), results up 2.3x (₹1,924cr → ₹4,341cr), and segment assets up 2.1x to ₹56,921cr, overtaking every other Tata segment. Adani Power has no renewables segment (that sits in sister company Adani Green). TRANSMISSION &amp; DISTRIBUTION: Tata Power's largest and steadiest segment — revenue grew ₹27,493cr → ₹41,339cr (FY22→FY26, boosted by the Odisha discoms) with consistently positive, regulated-return results (₹2,138cr → ₹4,308cr). Torrent's distribution business is economically similar (regulated, stable) but not separately reported. INDUSTRY CONTEXT: India's power demand grew ~7-8%/yr (CEA) over this period — Adani's generation growth (~13% CAGR) and Tata's renewables growth (~21% CAGR) both outpaced the sector, largely through acquisitions and capacity build-out respectively, while Tata's generation segment underperformed the sector.</t>
         </is>
       </c>
     </row>
@@ -11018,7 +10402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11051,114 +10435,95 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FY21</t>
+          <t>FY22</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13432.77</v>
+        <v>11211.03</v>
       </c>
       <c r="C2" t="n">
-        <v>5887.65</v>
+        <v>7748.9</v>
       </c>
       <c r="D2" t="n">
-        <v>16829.85</v>
+        <v>27493.17</v>
       </c>
       <c r="E2" t="n">
-        <v>25870.6</v>
+        <v>27221.78</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FY22</t>
+          <t>FY23</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11211.03</v>
+        <v>18211.35</v>
       </c>
       <c r="C3" t="n">
-        <v>7748.9</v>
+        <v>8196.91</v>
       </c>
       <c r="D3" t="n">
-        <v>27493.17</v>
+        <v>34529.36</v>
       </c>
       <c r="E3" t="n">
-        <v>27221.78</v>
+        <v>37895.85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FY23</t>
+          <t>FY24</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18211.35</v>
+        <v>19613.61</v>
       </c>
       <c r="C4" t="n">
-        <v>8196.91</v>
+        <v>10175.29</v>
       </c>
       <c r="D4" t="n">
-        <v>34529.36</v>
+        <v>36205.82</v>
       </c>
       <c r="E4" t="n">
-        <v>37895.85</v>
+        <v>50014.16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19613.61</v>
+        <v>19739.07</v>
       </c>
       <c r="C5" t="n">
-        <v>10175.29</v>
+        <v>9876.360000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>36205.82</v>
+        <v>39120.52</v>
       </c>
       <c r="E5" t="n">
-        <v>50014.16</v>
+        <v>56107.06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19739.07</v>
+        <v>11635.93</v>
       </c>
       <c r="C6" t="n">
-        <v>9876.360000000001</v>
+        <v>15027.82</v>
       </c>
       <c r="D6" t="n">
-        <v>39120.52</v>
+        <v>41338.59</v>
       </c>
       <c r="E6" t="n">
-        <v>56107.06</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>11635.93</v>
-      </c>
-      <c r="C7" t="n">
-        <v>15027.82</v>
-      </c>
-      <c r="D7" t="n">
-        <v>41338.59</v>
-      </c>
-      <c r="E7" t="n">
         <v>54240.52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Extend Adani BS/PL to full FY22-26 and fix incomplete Tata FY22 column
Adani_BS_Consolidated / Adani_PL_Consolidated: extended from FY22-23
only to the full FY22-FY26 window, extracted directly from all four
Adani Power Annual Report PDFs (FY22-23, FY23-24, FY24-25, FY25-26).
All Total Assets = Total Equity & Liabilities checks pass for every year.

Tata_BS_Consolidated: the FY2022 column was previously missing its
entire Liabilities section (Non-controlling Interests through
Regulatory Deferral Account) - pulled the FY21-22 Annual Report's own
Consolidated Balance Sheet to complete it. FY2022 now ties out exactly
(Total Assets = Total Equity and Liabilities = Rs 1,12,884.59cr).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dfAyzuD6csZoL9Xm9MRUV
</commit_message>
<xml_diff>
--- a/FADM_AdaniPower_Analysis.xlsx
+++ b/FADM_AdaniPower_Analysis.xlsx
@@ -8251,1006 +8251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>ADANI POWER LIMITED — Consolidated Balance Sheet</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="25" t="inlineStr">
-        <is>
-          <t>Source: Adani Power Ltd FY2022-23 Integrated Annual Report, 'Consolidated Balance Sheet as at 31st March, 2023' (repo file: AR_22088_ADANIPOWER_2022_2023). NOTE: an earlier draft sheet in this workbook ('Sheet5') showed Adani Power's STANDALONE balance sheet mislabeled — this sheet replaces it with the genuine consolidated figures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>Particulars (₹ crore)</t>
-        </is>
-      </c>
-      <c r="B4" s="27" t="inlineStr">
-        <is>
-          <t>As at 31-Mar-2023</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>As at 31-Mar-2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>ASSETS</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="11" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="28" t="inlineStr">
-        <is>
-          <t>Non-current Assets</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Property, Plant and Equipment</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="n">
-        <v>50543.8</v>
-      </c>
-      <c r="C7" s="30" t="n">
-        <v>53071.62</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Capital Work-in-Progress</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="n">
-        <v>12879.54</v>
-      </c>
-      <c r="C8" s="30" t="n">
-        <v>10269.74</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Investment Property</t>
-        </is>
-      </c>
-      <c r="B9" s="30" t="n">
-        <v>704.9400000000001</v>
-      </c>
-      <c r="C9" s="30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Goodwill</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="n">
-        <v>190.61</v>
-      </c>
-      <c r="C10" s="30" t="n">
-        <v>190.61</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Other Intangible Assets</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="n">
-        <v>12.03</v>
-      </c>
-      <c r="C11" s="30" t="n">
-        <v>11.98</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="29" t="inlineStr">
-        <is>
-          <t>Investments (Non-current)</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="n">
-        <v>42.51</v>
-      </c>
-      <c r="C12" s="30" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Other Financial Assets (Non-current)</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="n">
-        <v>779.71</v>
-      </c>
-      <c r="C13" s="30" t="n">
-        <v>856.04</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Other Non-current Assets</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="n">
-        <v>1115.13</v>
-      </c>
-      <c r="C14" s="30" t="n">
-        <v>1352.95</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Total Non-current Assets</t>
-        </is>
-      </c>
-      <c r="B15" s="31" t="n">
-        <v>66268.27</v>
-      </c>
-      <c r="C15" s="31" t="n">
-        <v>65752.95</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>Current Assets</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>Inventories</t>
-        </is>
-      </c>
-      <c r="B17" s="30" t="n">
-        <v>3075.2</v>
-      </c>
-      <c r="C17" s="30" t="n">
-        <v>2258.27</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>Investments (Current)</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="n">
-        <v>611.54</v>
-      </c>
-      <c r="C18" s="30" t="n">
-        <v>183.24</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="29" t="inlineStr">
-        <is>
-          <t>Trade Receivables</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="n">
-        <v>11529.36</v>
-      </c>
-      <c r="C19" s="30" t="n">
-        <v>9560.92</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>Cash and Cash Equivalents</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="n">
-        <v>349.23</v>
-      </c>
-      <c r="C20" s="30" t="n">
-        <v>782.37</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
-        <is>
-          <t>Bank Balances other than above</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="n">
-        <v>1524.42</v>
-      </c>
-      <c r="C21" s="30" t="n">
-        <v>1582.31</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="29" t="inlineStr">
-        <is>
-          <t>Loans (Current)</t>
-        </is>
-      </c>
-      <c r="B22" s="30" t="n">
-        <v>3.19</v>
-      </c>
-      <c r="C22" s="30" t="n">
-        <v>7.62</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>Other Financial Assets (Current)</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="n">
-        <v>557.5</v>
-      </c>
-      <c r="C23" s="30" t="n">
-        <v>308.28</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="29" t="inlineStr">
-        <is>
-          <t>Other Current Assets</t>
-        </is>
-      </c>
-      <c r="B24" s="30" t="n">
-        <v>1902.56</v>
-      </c>
-      <c r="C24" s="30" t="n">
-        <v>1545.06</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Total Current Assets</t>
-        </is>
-      </c>
-      <c r="B25" s="31" t="n">
-        <v>19553</v>
-      </c>
-      <c r="C25" s="31" t="n">
-        <v>16228.07</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL ASSETS</t>
-        </is>
-      </c>
-      <c r="B26" s="31" t="n">
-        <v>85821.27</v>
-      </c>
-      <c r="C26" s="31" t="n">
-        <v>81981.02</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="28" t="inlineStr">
-        <is>
-          <t>EQUITY AND LIABILITIES</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t>Equity Share Capital</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="n">
-        <v>3856.94</v>
-      </c>
-      <c r="C28" s="30" t="n">
-        <v>3856.94</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>Unsecured Perpetual Securities</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="n">
-        <v>13215</v>
-      </c>
-      <c r="C29" s="30" t="n">
-        <v>13215</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="29" t="inlineStr">
-        <is>
-          <t>Other Equity</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="n">
-        <v>12803.72</v>
-      </c>
-      <c r="C30" s="30" t="n">
-        <v>1631.5</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="29" t="inlineStr">
-        <is>
-          <t>Equity attributable to equity holders of the parent</t>
-        </is>
-      </c>
-      <c r="B31" s="30" t="n">
-        <v>29875.66</v>
-      </c>
-      <c r="C31" s="30" t="n">
-        <v>18703.44</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="29" t="inlineStr">
-        <is>
-          <t>Non-Controlling Interests</t>
-        </is>
-      </c>
-      <c r="B32" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="30" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>Total Equity</t>
-        </is>
-      </c>
-      <c r="B33" s="31" t="n">
-        <v>29875.66</v>
-      </c>
-      <c r="C33" s="31" t="n">
-        <v>18703.44</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t>Non-current Liabilities</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="n"/>
-      <c r="C34" s="11" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="29" t="inlineStr">
-        <is>
-          <t>Borrowings (Non-current)</t>
-        </is>
-      </c>
-      <c r="B35" s="30" t="n">
-        <v>33702.6</v>
-      </c>
-      <c r="C35" s="30" t="n">
-        <v>37871.32</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="29" t="inlineStr">
-        <is>
-          <t>Lease Liabilities (Non-current)</t>
-        </is>
-      </c>
-      <c r="B36" s="30" t="n">
-        <v>88.31999999999999</v>
-      </c>
-      <c r="C36" s="30" t="n">
-        <v>94.36</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="29" t="inlineStr">
-        <is>
-          <t>Other Financial Liabilities (Non-current)</t>
-        </is>
-      </c>
-      <c r="B37" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C37" s="30" t="n">
-        <v>960.37</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="29" t="inlineStr">
-        <is>
-          <t>Provisions (Non-current)</t>
-        </is>
-      </c>
-      <c r="B38" s="30" t="n">
-        <v>226.95</v>
-      </c>
-      <c r="C38" s="30" t="n">
-        <v>220.87</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="29" t="inlineStr">
-        <is>
-          <t>Deferred Tax Liabilities (Net)</t>
-        </is>
-      </c>
-      <c r="B39" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="30" t="n">
-        <v>2499.78</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="29" t="inlineStr">
-        <is>
-          <t>Other Non-current Liabilities</t>
-        </is>
-      </c>
-      <c r="B40" s="30" t="n">
-        <v>4183.15</v>
-      </c>
-      <c r="C40" s="30" t="n">
-        <v>4487.21</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>Total Non-current Liabilities</t>
-        </is>
-      </c>
-      <c r="B41" s="31" t="n">
-        <v>38201.02</v>
-      </c>
-      <c r="C41" s="31" t="n">
-        <v>46133.91</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="28" t="inlineStr">
-        <is>
-          <t>Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="n"/>
-      <c r="C42" s="11" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="29" t="inlineStr">
-        <is>
-          <t>Borrowings (Current)</t>
-        </is>
-      </c>
-      <c r="B43" s="30" t="n">
-        <v>8549.450000000001</v>
-      </c>
-      <c r="C43" s="30" t="n">
-        <v>10924.36</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="29" t="inlineStr">
-        <is>
-          <t>Lease Liabilities (Current)</t>
-        </is>
-      </c>
-      <c r="B44" s="30" t="n">
-        <v>9.16</v>
-      </c>
-      <c r="C44" s="30" t="n">
-        <v>8.390000000000001</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="29" t="inlineStr">
-        <is>
-          <t>Trade Payables — micro/small enterprises</t>
-        </is>
-      </c>
-      <c r="B45" s="30" t="n">
-        <v>95.76000000000001</v>
-      </c>
-      <c r="C45" s="30" t="n">
-        <v>57.59</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="29" t="inlineStr">
-        <is>
-          <t>Trade Payables — other creditors</t>
-        </is>
-      </c>
-      <c r="B46" s="30" t="n">
-        <v>2983.69</v>
-      </c>
-      <c r="C46" s="30" t="n">
-        <v>3450.62</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="29" t="inlineStr">
-        <is>
-          <t>Other Financial Liabilities (Current)</t>
-        </is>
-      </c>
-      <c r="B47" s="30" t="n">
-        <v>2461.58</v>
-      </c>
-      <c r="C47" s="30" t="n">
-        <v>1167.32</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="29" t="inlineStr">
-        <is>
-          <t>Other Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B48" s="30" t="n">
-        <v>3622.82</v>
-      </c>
-      <c r="C48" s="30" t="n">
-        <v>861.36</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="29" t="inlineStr">
-        <is>
-          <t>Provisions (Current)</t>
-        </is>
-      </c>
-      <c r="B49" s="30" t="n">
-        <v>21.64</v>
-      </c>
-      <c r="C49" s="30" t="n">
-        <v>28.71</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="29" t="inlineStr">
-        <is>
-          <t>Current Tax Liabilities (Net)</t>
-        </is>
-      </c>
-      <c r="B50" s="30" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="C50" s="30" t="n">
-        <v>645.3200000000001</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
-        <is>
-          <t>Total Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B51" s="31" t="n">
-        <v>17744.59</v>
-      </c>
-      <c r="C51" s="31" t="n">
-        <v>17143.67</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>Total Liabilities</t>
-        </is>
-      </c>
-      <c r="B52" s="31" t="n">
-        <v>55945.61</v>
-      </c>
-      <c r="C52" s="31" t="n">
-        <v>63277.58</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL EQUITY AND LIABILITIES</t>
-        </is>
-      </c>
-      <c r="B53" s="31" t="n">
-        <v>85821.27</v>
-      </c>
-      <c r="C53" s="31" t="n">
-        <v>81981.02</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>ADANI POWER LIMITED — Consolidated Statement of Profit and Loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="25" t="inlineStr">
-        <is>
-          <t>Source: Adani Power Ltd FY2022-23 Integrated Annual Report, 'Consolidated Statement of Profit and Loss for the year ended 31st March, 2023' (repo file: AR_22088_ADANIPOWER_2022_2023). NOTE: replaces an earlier draft sheet ('Consolidated Profit and loss st...') that was mislabeled and actually contained Adani Power's STANDALONE figures (PAT ₹10,246.15cr FY23) — the genuine consolidated PAT is ₹10,726.64cr.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>Particulars (₹ crore)</t>
-        </is>
-      </c>
-      <c r="B4" s="27" t="inlineStr">
-        <is>
-          <t>Year ended 31-Mar-2023</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>Year ended 31-Mar-2022</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="28" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="11" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Revenue from Operations</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="n">
-        <v>38773.3</v>
-      </c>
-      <c r="C6" s="30" t="n">
-        <v>27711.18</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Other Income</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="n">
-        <v>4267.22</v>
-      </c>
-      <c r="C7" s="30" t="n">
-        <v>3975.29</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Total Income</t>
-        </is>
-      </c>
-      <c r="B8" s="31" t="n">
-        <v>43040.52</v>
-      </c>
-      <c r="C8" s="31" t="n">
-        <v>31686.47</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="28" t="inlineStr">
-        <is>
-          <t>Expenses</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Fuel Cost</t>
-        </is>
-      </c>
-      <c r="B10" s="30" t="n">
-        <v>25480.85</v>
-      </c>
-      <c r="C10" s="30" t="n">
-        <v>14762.21</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Purchase of Stock-in-trade / Power for resale</t>
-        </is>
-      </c>
-      <c r="B11" s="30" t="n">
-        <v>214.14</v>
-      </c>
-      <c r="C11" s="30" t="n">
-        <v>545.5599999999999</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="29" t="inlineStr">
-        <is>
-          <t>Transmission Charges</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="n">
-        <v>519.61</v>
-      </c>
-      <c r="C12" s="30" t="n">
-        <v>642.77</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Employee Benefits Expense</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="n">
-        <v>569.99</v>
-      </c>
-      <c r="C13" s="30" t="n">
-        <v>470.31</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Finance Costs (net)</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="n">
-        <v>3333.5</v>
-      </c>
-      <c r="C14" s="30" t="n">
-        <v>4094.78</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="29" t="inlineStr">
-        <is>
-          <t>Depreciation and Amortisation Expense</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="n">
-        <v>3303.68</v>
-      </c>
-      <c r="C15" s="30" t="n">
-        <v>3117.54</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t>Other Expenses</t>
-        </is>
-      </c>
-      <c r="B16" s="30" t="n">
-        <v>1944.05</v>
-      </c>
-      <c r="C16" s="30" t="n">
-        <v>1476.17</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>Total Expenses</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n">
-        <v>35365.82</v>
-      </c>
-      <c r="C17" s="31" t="n">
-        <v>25109.34</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>Profit before tax and deferred tax (adj.)/recoverable from future tariff</t>
-        </is>
-      </c>
-      <c r="B18" s="30" t="n">
-        <v>7674.7</v>
-      </c>
-      <c r="C18" s="30" t="n">
-        <v>6577.13</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="29" t="inlineStr">
-        <is>
-          <t>Current Tax</t>
-        </is>
-      </c>
-      <c r="B19" s="30" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="C19" s="30" t="n">
-        <v>768.34</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>Tax credit adjusted relating to earlier years</t>
-        </is>
-      </c>
-      <c r="B20" s="30" t="n">
-        <v>-768.1799999999999</v>
-      </c>
-      <c r="C20" s="30" t="n">
-        <v>-0.11</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="29" t="inlineStr">
-        <is>
-          <t>Deferred Tax (credit)/charge (incl. earlier-year adj.)</t>
-        </is>
-      </c>
-      <c r="B21" s="30" t="n">
-        <v>-2499.77</v>
-      </c>
-      <c r="C21" s="30" t="n">
-        <v>976.5700000000001</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>Total Tax (Credit)/Expense</t>
-        </is>
-      </c>
-      <c r="B22" s="31" t="n">
-        <v>-3267.37</v>
-      </c>
-      <c r="C22" s="31" t="n">
-        <v>1744.8</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>Add: Deferred tax (adj.)/recoverable from future tariff (net of tax)</t>
-        </is>
-      </c>
-      <c r="B23" s="30" t="n">
-        <v>-215.43</v>
-      </c>
-      <c r="C23" s="30" t="n">
-        <v>79.25</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Profit for the Year (PAT)</t>
-        </is>
-      </c>
-      <c r="B24" s="31" t="n">
-        <v>10726.64</v>
-      </c>
-      <c r="C24" s="31" t="n">
-        <v>4911.58</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="29" t="inlineStr">
-        <is>
-          <t>Other Comprehensive Income, net of tax</t>
-        </is>
-      </c>
-      <c r="B25" s="30" t="n">
-        <v>33.74</v>
-      </c>
-      <c r="C25" s="30" t="n">
-        <v>43.63</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Total Comprehensive Income for the Year</t>
-        </is>
-      </c>
-      <c r="B26" s="31" t="n">
-        <v>10760.38</v>
-      </c>
-      <c r="C26" s="31" t="n">
-        <v>4955.21</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -9264,14 +8265,14 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>THE TATA POWER COMPANY LIMITED — Consolidated Balance Sheet</t>
+          <t>ADANI POWER LIMITED — Consolidated Balance Sheet</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="25" t="inlineStr">
         <is>
-          <t>Sources: Tata Power Integrated Annual Reports FY21-22 (AR_20052), FY23-24 (AR_24164) and FY25-26 (AR_29380) — 'Consolidated Balance Sheet' as at each year-end. Fills the FY24/FY25 gaps left blank in the team's original 'Tata Power' draft sheet; FY22/23/26 figures cross-checked and match.</t>
+          <t>Sources: Adani Power Ltd Integrated Annual Reports FY22-23 (AR_22088), FY23-24 (AR_24072), FY24-25 (ADANIPOWER-2025) and FY25-26 (AR_29298) — 'Consolidated Balance Sheet' as at each year-end. NOTE: an earlier draft sheet in this workbook ('Sheet5') showed Adani Power's STANDALONE balance sheet mislabeled as consolidated — this sheet replaces it with genuine consolidated figures across the full FY22-FY26 window.</t>
         </is>
       </c>
     </row>
@@ -9338,6 +8339,1666 @@
         </is>
       </c>
       <c r="B7" s="30" t="n">
+        <v>66814.60000000001</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>66707.23</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>62812.71</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>50543.8</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>53071.62</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Right-of-use Assets</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="n">
+        <v>2261.28</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>2319.82</v>
+      </c>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>Capital Work-in-Progress</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>35053.46</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>12104.42</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>925.12</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <v>12879.54</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>10269.74</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Investment Property</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>48.69</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>704.9400000000001</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Goodwill</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="n">
+        <v>204.52</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <v>204.52</v>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>190.61</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>190.61</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>190.61</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Other Intangible Assets</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>28.81</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>17.19</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>12.03</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>11.98</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Investments (Non-current)</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>59.51</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>42.51</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Loans (Non-current)</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Other Financial Assets (Non-current)</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>690.36</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>691.41</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>636.2</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>779.71</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>856.04</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Non-current Tax Assets (Net)</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>192.06</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <v>216.55</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>365.72</v>
+      </c>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>Deferred Tax Assets (Net)</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="n">
+        <v>811.39</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="30" t="n">
+        <v>376.34</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Other Non-current Assets</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>7410.97</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>4219</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>1418.95</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>1115.13</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>1352.95</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Total Non-current Assets</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n">
+        <v>113591.84</v>
+      </c>
+      <c r="C19" s="31" t="n">
+        <v>86588.34</v>
+      </c>
+      <c r="D19" s="31" t="n">
+        <v>66738.19</v>
+      </c>
+      <c r="E19" s="31" t="n">
+        <v>66268.27</v>
+      </c>
+      <c r="F19" s="31" t="n">
+        <v>65752.95</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Current Assets</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>Inventories</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="n">
+        <v>3623.48</v>
+      </c>
+      <c r="C21" s="30" t="n">
+        <v>3317.28</v>
+      </c>
+      <c r="D21" s="30" t="n">
+        <v>4142.1</v>
+      </c>
+      <c r="E21" s="30" t="n">
+        <v>3075.2</v>
+      </c>
+      <c r="F21" s="30" t="n">
+        <v>2258.27</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Investments (Current)</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="n">
+        <v>1491.35</v>
+      </c>
+      <c r="C22" s="30" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="D22" s="30" t="n">
+        <v>373.5</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>611.54</v>
+      </c>
+      <c r="F22" s="30" t="n">
+        <v>183.24</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="inlineStr">
+        <is>
+          <t>Trade Receivables</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="n">
+        <v>11791.37</v>
+      </c>
+      <c r="C23" s="30" t="n">
+        <v>13022.07</v>
+      </c>
+      <c r="D23" s="30" t="n">
+        <v>11677.48</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <v>11529.36</v>
+      </c>
+      <c r="F23" s="30" t="n">
+        <v>9560.92</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Cash and Cash Equivalents</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="n">
+        <v>927.88</v>
+      </c>
+      <c r="C24" s="30" t="n">
+        <v>319.86</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <v>1136.25</v>
+      </c>
+      <c r="E24" s="30" t="n">
+        <v>349.23</v>
+      </c>
+      <c r="F24" s="30" t="n">
+        <v>782.37</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Bank Balances other than above</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="n">
+        <v>5998.44</v>
+      </c>
+      <c r="C25" s="30" t="n">
+        <v>5800.02</v>
+      </c>
+      <c r="D25" s="30" t="n">
+        <v>6075.51</v>
+      </c>
+      <c r="E25" s="30" t="n">
+        <v>1524.42</v>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>1582.31</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Loans (Current)</t>
+        </is>
+      </c>
+      <c r="B26" s="30" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="C26" s="30" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="D26" s="30" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="E26" s="30" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F26" s="30" t="n">
+        <v>7.62</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Other Financial Assets (Current)</t>
+        </is>
+      </c>
+      <c r="B27" s="30" t="n">
+        <v>2161.97</v>
+      </c>
+      <c r="C27" s="30" t="n">
+        <v>887.51</v>
+      </c>
+      <c r="D27" s="30" t="n">
+        <v>435.82</v>
+      </c>
+      <c r="E27" s="30" t="n">
+        <v>557.5</v>
+      </c>
+      <c r="F27" s="30" t="n">
+        <v>308.28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Current Tax Assets (Net)</t>
+        </is>
+      </c>
+      <c r="B28" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="30" t="n">
+        <v>196.41</v>
+      </c>
+      <c r="D28" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="29" t="inlineStr">
+        <is>
+          <t>Other Current Assets</t>
+        </is>
+      </c>
+      <c r="B29" s="30" t="n">
+        <v>2682.6</v>
+      </c>
+      <c r="C29" s="30" t="n">
+        <v>1725.78</v>
+      </c>
+      <c r="D29" s="30" t="n">
+        <v>1742.43</v>
+      </c>
+      <c r="E29" s="30" t="n">
+        <v>1902.56</v>
+      </c>
+      <c r="F29" s="30" t="n">
+        <v>1545.06</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="n">
+        <v>28688.08</v>
+      </c>
+      <c r="C30" s="31" t="n">
+        <v>26313.45</v>
+      </c>
+      <c r="D30" s="31" t="n">
+        <v>25586.58</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <v>19553</v>
+      </c>
+      <c r="F30" s="31" t="n">
+        <v>16228.07</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>Assets Classified as Held for Sale</t>
+        </is>
+      </c>
+      <c r="B31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="30" t="n">
+        <v>15.78</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL ASSETS</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="n">
+        <v>142279.92</v>
+      </c>
+      <c r="C32" s="31" t="n">
+        <v>112917.57</v>
+      </c>
+      <c r="D32" s="31" t="n">
+        <v>92324.77</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <v>85821.27</v>
+      </c>
+      <c r="F32" s="31" t="n">
+        <v>81981.02</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>EQUITY AND LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>Equity Share Capital</t>
+        </is>
+      </c>
+      <c r="B34" s="30" t="n">
+        <v>3856.94</v>
+      </c>
+      <c r="C34" s="30" t="n">
+        <v>3856.94</v>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>3856.94</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <v>3856.94</v>
+      </c>
+      <c r="F34" s="30" t="n">
+        <v>3856.94</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>Instrument entirely Equity in nature / Unsecured Perpetual Securities</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="30" t="n">
+        <v>3056.92</v>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>7315</v>
+      </c>
+      <c r="E35" s="30" t="n">
+        <v>13215</v>
+      </c>
+      <c r="F35" s="30" t="n">
+        <v>13215</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>Other Equity</t>
+        </is>
+      </c>
+      <c r="B36" s="30" t="n">
+        <v>61079.94</v>
+      </c>
+      <c r="C36" s="30" t="n">
+        <v>49433.23</v>
+      </c>
+      <c r="D36" s="30" t="n">
+        <v>31973.09</v>
+      </c>
+      <c r="E36" s="30" t="n">
+        <v>12803.72</v>
+      </c>
+      <c r="F36" s="30" t="n">
+        <v>1631.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Equity attributable to equity holders of the parent</t>
+        </is>
+      </c>
+      <c r="B37" s="30" t="n">
+        <v>64936.88</v>
+      </c>
+      <c r="C37" s="30" t="n">
+        <v>56347.09</v>
+      </c>
+      <c r="D37" s="30" t="n">
+        <v>43145.03</v>
+      </c>
+      <c r="E37" s="30" t="n">
+        <v>29875.66</v>
+      </c>
+      <c r="F37" s="30" t="n">
+        <v>18703.44</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Non-Controlling Interests</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="n">
+        <v>1465.04</v>
+      </c>
+      <c r="C38" s="30" t="n">
+        <v>1326.47</v>
+      </c>
+      <c r="D38" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>Total Equity</t>
+        </is>
+      </c>
+      <c r="B39" s="31" t="n">
+        <v>66401.92</v>
+      </c>
+      <c r="C39" s="31" t="n">
+        <v>57673.56</v>
+      </c>
+      <c r="D39" s="31" t="n">
+        <v>43145.03</v>
+      </c>
+      <c r="E39" s="31" t="n">
+        <v>29875.66</v>
+      </c>
+      <c r="F39" s="31" t="n">
+        <v>18703.44</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="28" t="inlineStr">
+        <is>
+          <t>Non-current Liabilities</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>Borrowings (Non-current)</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="n">
+        <v>42829.6</v>
+      </c>
+      <c r="C41" s="30" t="n">
+        <v>27646.96</v>
+      </c>
+      <c r="D41" s="30" t="n">
+        <v>26595.01</v>
+      </c>
+      <c r="E41" s="30" t="n">
+        <v>33702.6</v>
+      </c>
+      <c r="F41" s="30" t="n">
+        <v>37871.32</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>Lease Liabilities (Non-current)</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="n">
+        <v>1049.27</v>
+      </c>
+      <c r="C42" s="30" t="n">
+        <v>1094.04</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>143.11</v>
+      </c>
+      <c r="E42" s="30" t="n">
+        <v>88.31999999999999</v>
+      </c>
+      <c r="F42" s="30" t="n">
+        <v>94.36</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>Other Financial Liabilities (Non-current)</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="n">
+        <v>185.69</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E43" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="30" t="n">
+        <v>960.37</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>Provisions (Non-current)</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="n">
+        <v>359.9</v>
+      </c>
+      <c r="C44" s="30" t="n">
+        <v>339.64</v>
+      </c>
+      <c r="D44" s="30" t="n">
+        <v>237.45</v>
+      </c>
+      <c r="E44" s="30" t="n">
+        <v>226.95</v>
+      </c>
+      <c r="F44" s="30" t="n">
+        <v>220.87</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="29" t="inlineStr">
+        <is>
+          <t>Deferred Tax Liabilities (Net)</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="n">
+        <v>5827.15</v>
+      </c>
+      <c r="C45" s="30" t="n">
+        <v>4022.73</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>315.8</v>
+      </c>
+      <c r="E45" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="30" t="n">
+        <v>2499.78</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>Other Non-current Liabilities</t>
+        </is>
+      </c>
+      <c r="B46" s="30" t="n">
+        <v>5298.18</v>
+      </c>
+      <c r="C46" s="30" t="n">
+        <v>5698.48</v>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>6098.63</v>
+      </c>
+      <c r="E46" s="30" t="n">
+        <v>4183.15</v>
+      </c>
+      <c r="F46" s="30" t="n">
+        <v>4487.21</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Total Non-current Liabilities</t>
+        </is>
+      </c>
+      <c r="B47" s="31" t="n">
+        <v>55549.79</v>
+      </c>
+      <c r="C47" s="31" t="n">
+        <v>38803.02</v>
+      </c>
+      <c r="D47" s="31" t="n">
+        <v>33391.07</v>
+      </c>
+      <c r="E47" s="31" t="n">
+        <v>38201.02</v>
+      </c>
+      <c r="F47" s="31" t="n">
+        <v>46133.91</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t>Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="29" t="inlineStr">
+        <is>
+          <t>Borrowings (Current)</t>
+        </is>
+      </c>
+      <c r="B49" s="30" t="n">
+        <v>10725.94</v>
+      </c>
+      <c r="C49" s="30" t="n">
+        <v>10687.92</v>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>7861.85</v>
+      </c>
+      <c r="E49" s="30" t="n">
+        <v>8549.450000000001</v>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>10924.36</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="29" t="inlineStr">
+        <is>
+          <t>Lease Liabilities (Current)</t>
+        </is>
+      </c>
+      <c r="B50" s="30" t="n">
+        <v>65.48</v>
+      </c>
+      <c r="C50" s="30" t="n">
+        <v>65.95</v>
+      </c>
+      <c r="D50" s="30" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="E50" s="30" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="F50" s="30" t="n">
+        <v>8.390000000000001</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>Trade Payables — micro/small enterprises</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="n">
+        <v>183.98</v>
+      </c>
+      <c r="C51" s="30" t="n">
+        <v>215.73</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>141.93</v>
+      </c>
+      <c r="E51" s="30" t="n">
+        <v>95.76000000000001</v>
+      </c>
+      <c r="F51" s="30" t="n">
+        <v>57.59</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>Trade Payables — other creditors</t>
+        </is>
+      </c>
+      <c r="B52" s="30" t="n">
+        <v>2656.55</v>
+      </c>
+      <c r="C52" s="30" t="n">
+        <v>2761.93</v>
+      </c>
+      <c r="D52" s="30" t="n">
+        <v>3494.37</v>
+      </c>
+      <c r="E52" s="30" t="n">
+        <v>2983.69</v>
+      </c>
+      <c r="F52" s="30" t="n">
+        <v>3450.62</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="inlineStr">
+        <is>
+          <t>Other Financial Liabilities (Current)</t>
+        </is>
+      </c>
+      <c r="B53" s="30" t="n">
+        <v>4049.65</v>
+      </c>
+      <c r="C53" s="30" t="n">
+        <v>1230.62</v>
+      </c>
+      <c r="D53" s="30" t="n">
+        <v>2089.8</v>
+      </c>
+      <c r="E53" s="30" t="n">
+        <v>2461.58</v>
+      </c>
+      <c r="F53" s="30" t="n">
+        <v>1167.32</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B54" s="30" t="n">
+        <v>994.38</v>
+      </c>
+      <c r="C54" s="30" t="n">
+        <v>1348.74</v>
+      </c>
+      <c r="D54" s="30" t="n">
+        <v>2159.44</v>
+      </c>
+      <c r="E54" s="30" t="n">
+        <v>3622.82</v>
+      </c>
+      <c r="F54" s="30" t="n">
+        <v>861.36</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="29" t="inlineStr">
+        <is>
+          <t>Provisions (Current)</t>
+        </is>
+      </c>
+      <c r="B55" s="30" t="n">
+        <v>96.95999999999999</v>
+      </c>
+      <c r="C55" s="30" t="n">
+        <v>70.23999999999999</v>
+      </c>
+      <c r="D55" s="30" t="n">
+        <v>25.69</v>
+      </c>
+      <c r="E55" s="30" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="F55" s="30" t="n">
+        <v>28.71</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>Current Tax Liabilities (Net)</t>
+        </is>
+      </c>
+      <c r="B56" s="30" t="n">
+        <v>1555.27</v>
+      </c>
+      <c r="C56" s="30" t="n">
+        <v>59.86</v>
+      </c>
+      <c r="D56" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="30" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F56" s="30" t="n">
+        <v>645.3200000000001</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B57" s="31" t="n">
+        <v>20328.21</v>
+      </c>
+      <c r="C57" s="31" t="n">
+        <v>16440.99</v>
+      </c>
+      <c r="D57" s="31" t="n">
+        <v>15788.67</v>
+      </c>
+      <c r="E57" s="31" t="n">
+        <v>17744.59</v>
+      </c>
+      <c r="F57" s="31" t="n">
+        <v>17143.67</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="n">
+        <v>75878</v>
+      </c>
+      <c r="C58" s="31" t="n">
+        <v>55244.01</v>
+      </c>
+      <c r="D58" s="31" t="n">
+        <v>49179.74</v>
+      </c>
+      <c r="E58" s="31" t="n">
+        <v>55945.61</v>
+      </c>
+      <c r="F58" s="31" t="n">
+        <v>63277.58</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL EQUITY AND LIABILITIES</t>
+        </is>
+      </c>
+      <c r="B59" s="31" t="n">
+        <v>142279.92</v>
+      </c>
+      <c r="C59" s="31" t="n">
+        <v>112917.57</v>
+      </c>
+      <c r="D59" s="31" t="n">
+        <v>92324.77</v>
+      </c>
+      <c r="E59" s="31" t="n">
+        <v>85821.27</v>
+      </c>
+      <c r="F59" s="31" t="n">
+        <v>81981.02</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ADANI POWER LIMITED — Consolidated Statement of Profit and Loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Sources: Adani Power Ltd Integrated Annual Reports FY22-23, FY23-24, FY24-25 and FY25-26 — 'Consolidated Statement of Profit and Loss' for each year ended. NOTE: replaces an earlier draft sheet ('Consolidated Profit and loss st...') that was mislabeled and actually contained Adani Power's STANDALONE figures (PAT ₹10,246.15cr FY23) — the genuine consolidated PAT is ₹10,726.64cr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Particulars (₹ crore)</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>FY 2025-26</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>FY 2024-25</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>FY 2023-24</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>FY 2022-23</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>FY 2021-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Revenue from Operations</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="n">
+        <v>54240.52</v>
+      </c>
+      <c r="C6" s="30" t="n">
+        <v>56203.09</v>
+      </c>
+      <c r="D6" s="30" t="n">
+        <v>50351.25</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <v>38773.3</v>
+      </c>
+      <c r="F6" s="30" t="n">
+        <v>27711.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="n">
+        <v>3624.76</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>2702.74</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>9930.23</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <v>4267.22</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>3975.29</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Total Income</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="n">
+        <v>57865.28</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>58905.83</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>60281.48</v>
+      </c>
+      <c r="E8" s="31" t="n">
+        <v>43040.52</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>31686.47</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Expenses</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Fuel Cost</t>
+        </is>
+      </c>
+      <c r="B10" s="30" t="n">
+        <v>29168.02</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>30273.25</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>28452.64</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <v>25480.85</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>14762.21</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Purchase of Stock-in-trade / Power for resale</t>
+        </is>
+      </c>
+      <c r="B11" s="30" t="n">
+        <v>209.66</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <v>356.99</v>
+      </c>
+      <c r="D11" s="30" t="n">
+        <v>222.26</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <v>214.14</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>545.5599999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Transmission Charges</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="n">
+        <v>557.42</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>459.09</v>
+      </c>
+      <c r="D12" s="30" t="n">
+        <v>503.99</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>519.61</v>
+      </c>
+      <c r="F12" s="30" t="n">
+        <v>642.77</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Employee Benefits Expense</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>855.1799999999999</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>784.4</v>
+      </c>
+      <c r="D13" s="30" t="n">
+        <v>643.7</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>569.99</v>
+      </c>
+      <c r="F13" s="30" t="n">
+        <v>470.31</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Finance Costs (net)</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="n">
+        <v>3366.83</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>3339.79</v>
+      </c>
+      <c r="D14" s="30" t="n">
+        <v>3388.09</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <v>3333.5</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>4094.78</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Depreciation and Amortisation Expense</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>4564.53</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>4308.88</v>
+      </c>
+      <c r="D15" s="30" t="n">
+        <v>3931.33</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>3303.68</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>3117.54</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Other Expenses</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>3644.13</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <v>3023.92</v>
+      </c>
+      <c r="D16" s="30" t="n">
+        <v>2347.96</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <v>1944.05</v>
+      </c>
+      <c r="F16" s="30" t="n">
+        <v>1476.17</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Total Expenses</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n">
+        <v>42365.77</v>
+      </c>
+      <c r="C17" s="31" t="n">
+        <v>42546.32</v>
+      </c>
+      <c r="D17" s="31" t="n">
+        <v>39489.97</v>
+      </c>
+      <c r="E17" s="31" t="n">
+        <v>35365.82</v>
+      </c>
+      <c r="F17" s="31" t="n">
+        <v>25109.34</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Profit before share of JV profit and tax</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>15499.51</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>16359.51</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>20791.51</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <v>7674.7</v>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>6577.13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Total Tax Expense/(Credit)</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="n">
+        <v>2528.43</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>3609.9</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>-37.28</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <v>-3267.37</v>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>1744.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Add: Deferred tax (adj.)/recoverable from future tariff (net of tax)</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="30" t="n">
+        <v>-215.43</v>
+      </c>
+      <c r="F20" s="30" t="n">
+        <v>79.25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Profit for the Year (PAT, consolidated)</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n">
+        <v>12971.08</v>
+      </c>
+      <c r="C21" s="31" t="n">
+        <v>12749.61</v>
+      </c>
+      <c r="D21" s="31" t="n">
+        <v>20828.79</v>
+      </c>
+      <c r="E21" s="31" t="n">
+        <v>10726.64</v>
+      </c>
+      <c r="F21" s="31" t="n">
+        <v>4911.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="inlineStr">
+        <is>
+          <t>Other Comprehensive Income, net of tax</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="n">
+        <v>19.67</v>
+      </c>
+      <c r="C22" s="30" t="n">
+        <v>-2.69</v>
+      </c>
+      <c r="D22" s="30" t="n">
+        <v>-27.49</v>
+      </c>
+      <c r="E22" s="30" t="n">
+        <v>33.74</v>
+      </c>
+      <c r="F22" s="30" t="n">
+        <v>43.63</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Total Comprehensive Income for the Year</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="n">
+        <v>12990.75</v>
+      </c>
+      <c r="C23" s="31" t="n">
+        <v>12746.92</v>
+      </c>
+      <c r="D23" s="31" t="n">
+        <v>20801.3</v>
+      </c>
+      <c r="E23" s="31" t="n">
+        <v>10760.38</v>
+      </c>
+      <c r="F23" s="31" t="n">
+        <v>4955.21</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>THE TATA POWER COMPANY LIMITED — Consolidated Balance Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Sources: Tata Power Integrated Annual Reports FY21-22 (AR_20052), FY23-24 (AR_24164) and FY25-26 (AR_29380) — 'Consolidated Balance Sheet' as at each year-end. Fills the FY24/FY25 gaps left blank in the team's original 'Tata Power' draft sheet; FY22/23/26 figures cross-checked and match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>Particulars (₹ crore)</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Mar-2025</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Mar-2024</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Mar-2023</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Mar-2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>ASSETS</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Non-current Assets</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="11" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Property, Plant and Equipment</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="n">
         <v>78870.53999999999</v>
       </c>
       <c r="C7" s="30" t="n">
@@ -10121,7 +10782,9 @@
       <c r="E43" s="30" t="n">
         <v>5416.69</v>
       </c>
-      <c r="F43" s="11" t="n"/>
+      <c r="F43" s="30" t="n">
+        <v>3586.9</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
@@ -10141,7 +10804,9 @@
       <c r="E44" s="31" t="n">
         <v>34204.12</v>
       </c>
-      <c r="F44" s="32" t="n"/>
+      <c r="F44" s="31" t="n">
+        <v>26028.46</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="28" t="inlineStr">
@@ -10173,7 +10838,9 @@
       <c r="E46" s="30" t="n">
         <v>30708.49</v>
       </c>
-      <c r="F46" s="11" t="n"/>
+      <c r="F46" s="30" t="n">
+        <v>32729.7</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="29" t="inlineStr">
@@ -10193,359 +10860,419 @@
       <c r="E47" s="30" t="n">
         <v>3510.7</v>
       </c>
-      <c r="F47" s="11" t="n"/>
+      <c r="F47" s="30" t="n">
+        <v>3207.79</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="29" t="inlineStr">
         <is>
-          <t>Other Financial Liabilities (Non-current)</t>
-        </is>
-      </c>
-      <c r="B48" s="30" t="n">
-        <v>694.64</v>
-      </c>
-      <c r="C48" s="30" t="n">
-        <v>674.12</v>
-      </c>
-      <c r="D48" s="30" t="n">
-        <v>1507.55</v>
-      </c>
-      <c r="E48" s="30" t="n">
-        <v>1410.4</v>
-      </c>
-      <c r="F48" s="11" t="n"/>
+          <t>Trade Payables (Non-current)</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="11" t="n"/>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="29" t="inlineStr">
         <is>
-          <t>Provisions (Non-current)</t>
+          <t>Other Financial Liabilities (Non-current)</t>
         </is>
       </c>
       <c r="B49" s="30" t="n">
-        <v>3213.85</v>
+        <v>694.64</v>
       </c>
       <c r="C49" s="30" t="n">
-        <v>2548.69</v>
+        <v>674.12</v>
       </c>
       <c r="D49" s="30" t="n">
-        <v>1865.08</v>
+        <v>1507.55</v>
       </c>
       <c r="E49" s="30" t="n">
-        <v>1420.02</v>
-      </c>
-      <c r="F49" s="11" t="n"/>
+        <v>1410.4</v>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>1156.56</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="29" t="inlineStr">
         <is>
-          <t>Deferred Tax Liabilities (Net)</t>
-        </is>
-      </c>
-      <c r="B50" s="30" t="n">
-        <v>4807.88</v>
-      </c>
-      <c r="C50" s="30" t="n">
-        <v>4104.12</v>
-      </c>
-      <c r="D50" s="30" t="n">
-        <v>2772.33</v>
-      </c>
-      <c r="E50" s="30" t="n">
-        <v>1919.37</v>
-      </c>
-      <c r="F50" s="11" t="n"/>
+          <t>Non-current Tax Liabilities (Net)</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="30" t="n">
+        <v>3.03</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="29" t="inlineStr">
         <is>
+          <t>Provisions (Non-current)</t>
+        </is>
+      </c>
+      <c r="B51" s="30" t="n">
+        <v>3213.85</v>
+      </c>
+      <c r="C51" s="30" t="n">
+        <v>2548.69</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>1865.08</v>
+      </c>
+      <c r="E51" s="30" t="n">
+        <v>1420.02</v>
+      </c>
+      <c r="F51" s="30" t="n">
+        <v>1218.18</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>Deferred Tax Liabilities (Net)</t>
+        </is>
+      </c>
+      <c r="B52" s="30" t="n">
+        <v>4807.88</v>
+      </c>
+      <c r="C52" s="30" t="n">
+        <v>4104.12</v>
+      </c>
+      <c r="D52" s="30" t="n">
+        <v>2772.33</v>
+      </c>
+      <c r="E52" s="30" t="n">
+        <v>1919.37</v>
+      </c>
+      <c r="F52" s="30" t="n">
+        <v>1033.3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="29" t="inlineStr">
+        <is>
           <t>Other Non-current Liabilities</t>
         </is>
       </c>
-      <c r="B51" s="30" t="n">
+      <c r="B53" s="30" t="n">
         <v>13411.97</v>
       </c>
-      <c r="C51" s="30" t="n">
+      <c r="C53" s="30" t="n">
         <v>12930.57</v>
       </c>
-      <c r="D51" s="30" t="n">
+      <c r="D53" s="30" t="n">
         <v>11973.08</v>
       </c>
-      <c r="E51" s="30" t="n">
+      <c r="E53" s="30" t="n">
         <v>9847.82</v>
       </c>
-      <c r="F51" s="11" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="15" t="inlineStr">
+      <c r="F53" s="30" t="n">
+        <v>8139.29</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>Total Non-current Liabilities</t>
         </is>
       </c>
-      <c r="B52" s="31" t="n">
+      <c r="B54" s="31" t="n">
         <v>88286.85000000001</v>
       </c>
-      <c r="C52" s="31" t="n">
+      <c r="C54" s="31" t="n">
         <v>68583.42999999999</v>
       </c>
-      <c r="D52" s="31" t="n">
+      <c r="D54" s="31" t="n">
         <v>59252.77</v>
       </c>
-      <c r="E52" s="31" t="n">
+      <c r="E54" s="31" t="n">
         <v>48816.8</v>
       </c>
-      <c r="F52" s="32" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="28" t="inlineStr">
+      <c r="F54" s="31" t="n">
+        <v>47487.85</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="28" t="inlineStr">
         <is>
           <t>Current Liabilities</t>
         </is>
       </c>
-      <c r="B53" s="11" t="n"/>
-      <c r="C53" s="11" t="n"/>
-      <c r="D53" s="11" t="n"/>
-      <c r="E53" s="11" t="n"/>
-      <c r="F53" s="11" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="29" t="inlineStr">
-        <is>
-          <t>Borrowings (Current)</t>
-        </is>
-      </c>
-      <c r="B54" s="30" t="n">
-        <v>9513.82</v>
-      </c>
-      <c r="C54" s="30" t="n">
-        <v>14015.84</v>
-      </c>
-      <c r="D54" s="30" t="n">
-        <v>12087.56</v>
-      </c>
-      <c r="E54" s="30" t="n">
-        <v>18265.94</v>
-      </c>
-      <c r="F54" s="11" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="29" t="inlineStr">
-        <is>
-          <t>Lease Liabilities (Current)</t>
-        </is>
-      </c>
-      <c r="B55" s="30" t="n">
-        <v>468.94</v>
-      </c>
-      <c r="C55" s="30" t="n">
-        <v>524.03</v>
-      </c>
-      <c r="D55" s="30" t="n">
-        <v>467.16</v>
-      </c>
-      <c r="E55" s="30" t="n">
-        <v>437.87</v>
-      </c>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
       <c r="F55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="29" t="inlineStr">
         <is>
-          <t>Trade Payables — micro/small enterprises</t>
+          <t>Borrowings (Current)</t>
         </is>
       </c>
       <c r="B56" s="30" t="n">
-        <v>809.84</v>
+        <v>9513.82</v>
       </c>
       <c r="C56" s="30" t="n">
-        <v>784.21</v>
+        <v>14015.84</v>
       </c>
       <c r="D56" s="30" t="n">
-        <v>870</v>
+        <v>12087.56</v>
       </c>
       <c r="E56" s="30" t="n">
-        <v>537.6</v>
-      </c>
-      <c r="F56" s="11" t="n"/>
+        <v>18265.94</v>
+      </c>
+      <c r="F56" s="30" t="n">
+        <v>14860.3</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="29" t="inlineStr">
         <is>
-          <t>Trade Payables — other creditors</t>
+          <t>Lease Liabilities (Current)</t>
         </is>
       </c>
       <c r="B57" s="30" t="n">
-        <v>6328.39</v>
+        <v>468.94</v>
       </c>
       <c r="C57" s="30" t="n">
-        <v>8070.34</v>
+        <v>524.03</v>
       </c>
       <c r="D57" s="30" t="n">
-        <v>8451.370000000001</v>
+        <v>467.16</v>
       </c>
       <c r="E57" s="30" t="n">
-        <v>6869.6</v>
-      </c>
-      <c r="F57" s="11" t="n"/>
+        <v>437.87</v>
+      </c>
+      <c r="F57" s="30" t="n">
+        <v>397.33</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="29" t="inlineStr">
         <is>
-          <t>Other Financial Liabilities (Current)</t>
+          <t>Trade Payables — micro/small enterprises</t>
         </is>
       </c>
       <c r="B58" s="30" t="n">
-        <v>13897.6</v>
+        <v>809.84</v>
       </c>
       <c r="C58" s="30" t="n">
-        <v>12427.03</v>
+        <v>784.21</v>
       </c>
       <c r="D58" s="30" t="n">
-        <v>14796.16</v>
+        <v>870</v>
       </c>
       <c r="E58" s="30" t="n">
-        <v>13150.77</v>
+        <v>537.6</v>
       </c>
       <c r="F58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="29" t="inlineStr">
         <is>
-          <t>Provisions (Current)</t>
+          <t>Trade Payables — other creditors / total</t>
         </is>
       </c>
       <c r="B59" s="30" t="n">
-        <v>680.4400000000001</v>
+        <v>6328.39</v>
       </c>
       <c r="C59" s="30" t="n">
-        <v>437.56</v>
+        <v>8070.34</v>
       </c>
       <c r="D59" s="30" t="n">
-        <v>294.34</v>
+        <v>8451.370000000001</v>
       </c>
       <c r="E59" s="30" t="n">
-        <v>311.07</v>
-      </c>
-      <c r="F59" s="11" t="n"/>
+        <v>6869.6</v>
+      </c>
+      <c r="F59" s="30" t="n">
+        <v>10459.6</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="29" t="inlineStr">
         <is>
-          <t>Current Tax Liabilities (Net)</t>
+          <t>Other Financial Liabilities (Current)</t>
         </is>
       </c>
       <c r="B60" s="30" t="n">
-        <v>185.42</v>
+        <v>13897.6</v>
       </c>
       <c r="C60" s="30" t="n">
-        <v>208.2</v>
+        <v>12427.03</v>
       </c>
       <c r="D60" s="30" t="n">
-        <v>291.54</v>
+        <v>14796.16</v>
       </c>
       <c r="E60" s="30" t="n">
-        <v>217.96</v>
-      </c>
-      <c r="F60" s="11" t="n"/>
+        <v>13150.77</v>
+      </c>
+      <c r="F60" s="30" t="n">
+        <v>9631.959999999999</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="29" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Provisions (Current)</t>
         </is>
       </c>
       <c r="B61" s="30" t="n">
-        <v>3691.15</v>
+        <v>680.4400000000001</v>
       </c>
       <c r="C61" s="30" t="n">
-        <v>3672.38</v>
+        <v>437.56</v>
       </c>
       <c r="D61" s="30" t="n">
-        <v>3879.84</v>
+        <v>294.34</v>
       </c>
       <c r="E61" s="30" t="n">
-        <v>4188.41</v>
-      </c>
-      <c r="F61" s="11" t="n"/>
+        <v>311.07</v>
+      </c>
+      <c r="F61" s="30" t="n">
+        <v>344.82</v>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="15" t="inlineStr">
-        <is>
-          <t>Total Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B62" s="31" t="n">
-        <v>39223.57</v>
-      </c>
-      <c r="C62" s="31" t="n">
-        <v>45269.52</v>
-      </c>
-      <c r="D62" s="31" t="n">
-        <v>41137.97</v>
-      </c>
-      <c r="E62" s="31" t="n">
-        <v>43979.22</v>
-      </c>
-      <c r="F62" s="32" t="n"/>
+      <c r="A62" s="29" t="inlineStr">
+        <is>
+          <t>Current Tax Liabilities (Net)</t>
+        </is>
+      </c>
+      <c r="B62" s="30" t="n">
+        <v>185.42</v>
+      </c>
+      <c r="C62" s="30" t="n">
+        <v>208.2</v>
+      </c>
+      <c r="D62" s="30" t="n">
+        <v>291.54</v>
+      </c>
+      <c r="E62" s="30" t="n">
+        <v>217.96</v>
+      </c>
+      <c r="F62" s="30" t="n">
+        <v>147</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="29" t="inlineStr">
         <is>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B63" s="30" t="n">
+        <v>3691.15</v>
+      </c>
+      <c r="C63" s="30" t="n">
+        <v>3672.38</v>
+      </c>
+      <c r="D63" s="30" t="n">
+        <v>3879.84</v>
+      </c>
+      <c r="E63" s="30" t="n">
+        <v>4188.41</v>
+      </c>
+      <c r="F63" s="30" t="n">
+        <v>2779.08</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B64" s="31" t="n">
+        <v>39223.57</v>
+      </c>
+      <c r="C64" s="31" t="n">
+        <v>45269.52</v>
+      </c>
+      <c r="D64" s="31" t="n">
+        <v>41137.97</v>
+      </c>
+      <c r="E64" s="31" t="n">
+        <v>43979.22</v>
+      </c>
+      <c r="F64" s="31" t="n">
+        <v>38620.09</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="29" t="inlineStr">
+        <is>
           <t>Liabilities re: Assets Held For Sale</t>
         </is>
       </c>
-      <c r="B63" s="30" t="n">
+      <c r="B65" s="30" t="n">
         <v>114.24</v>
       </c>
-      <c r="C63" s="30" t="n">
+      <c r="C65" s="30" t="n">
         <v>113.56</v>
       </c>
-      <c r="D63" s="30" t="n">
+      <c r="D65" s="30" t="n">
         <v>113.56</v>
       </c>
-      <c r="E63" s="30" t="n">
+      <c r="E65" s="30" t="n">
         <v>113.56</v>
       </c>
-      <c r="F63" s="11" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="29" t="inlineStr">
+      <c r="F65" s="30" t="n">
+        <v>113.56</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="29" t="inlineStr">
         <is>
           <t>Regulatory Deferral Account — Liability</t>
         </is>
       </c>
-      <c r="B64" s="30" t="n">
+      <c r="B66" s="30" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="C64" s="30" t="n">
+      <c r="C66" s="30" t="n">
         <v>138.74</v>
       </c>
-      <c r="D64" s="30" t="n">
+      <c r="D66" s="30" t="n">
         <v>716.42</v>
       </c>
-      <c r="E64" s="30" t="n">
+      <c r="E66" s="30" t="n">
         <v>1235.34</v>
       </c>
-      <c r="F64" s="11" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="15" t="inlineStr">
+      <c r="F66" s="30" t="n">
+        <v>634.63</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>TOTAL EQUITY AND LIABILITIES</t>
         </is>
       </c>
-      <c r="B65" s="31" t="n">
+      <c r="B67" s="31" t="n">
         <v>175171.78</v>
       </c>
-      <c r="C65" s="31" t="n">
+      <c r="C67" s="31" t="n">
         <v>156711.29</v>
       </c>
-      <c r="D65" s="31" t="n">
+      <c r="D67" s="31" t="n">
         <v>139553.49</v>
       </c>
-      <c r="E65" s="31" t="n">
+      <c r="E67" s="31" t="n">
         <v>128349.04</v>
       </c>
-      <c r="F65" s="31" t="n">
+      <c r="F67" s="31" t="n">
         <v>112884.59</v>
       </c>
     </row>

</xml_diff>